<commit_message>
Fix formula bugs and clean up code review issues
</commit_message>
<xml_diff>
--- a/manufacturing-warehouse-planning/仓库规划库存需求计算模板.xlsx
+++ b/manufacturing-warehouse-planning/仓库规划库存需求计算模板.xlsx
@@ -2813,7 +2813,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="9" t="n"/>
-      <c r="H4" s="11">
+      <c r="H4" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -2859,7 +2859,7 @@
         <v>15</v>
       </c>
       <c r="G5" s="9" t="n"/>
-      <c r="H5" s="11">
+      <c r="H5" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -2905,7 +2905,7 @@
         <v>15</v>
       </c>
       <c r="G6" s="9" t="n"/>
-      <c r="H6" s="11">
+      <c r="H6" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -2951,7 +2951,7 @@
         <v>15</v>
       </c>
       <c r="G7" s="9" t="n"/>
-      <c r="H7" s="11">
+      <c r="H7" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -2997,7 +2997,7 @@
         <v>15</v>
       </c>
       <c r="G8" s="9" t="n"/>
-      <c r="H8" s="11">
+      <c r="H8" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3043,7 +3043,7 @@
         <v>15</v>
       </c>
       <c r="G9" s="9" t="n"/>
-      <c r="H9" s="11">
+      <c r="H9" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3089,7 +3089,7 @@
         <v>15</v>
       </c>
       <c r="G10" s="9" t="n"/>
-      <c r="H10" s="11">
+      <c r="H10" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3135,7 +3135,7 @@
         <v>15</v>
       </c>
       <c r="G11" s="9" t="n"/>
-      <c r="H11" s="11">
+      <c r="H11" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="F12" s="9" t="n"/>
       <c r="G12" s="9" t="n"/>
-      <c r="H12" s="11">
+      <c r="H12" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F13" s="9" t="n"/>
       <c r="G13" s="9" t="n"/>
-      <c r="H13" s="11">
+      <c r="H13" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="F14" s="9" t="n"/>
       <c r="G14" s="9" t="n"/>
-      <c r="H14" s="11">
+      <c r="H14" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3311,7 +3311,7 @@
       </c>
       <c r="F15" s="9" t="n"/>
       <c r="G15" s="9" t="n"/>
-      <c r="H15" s="11">
+      <c r="H15" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="F16" s="9" t="n"/>
       <c r="G16" s="9" t="n"/>
-      <c r="H16" s="11">
+      <c r="H16" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="F17" s="9" t="n"/>
       <c r="G17" s="9" t="n"/>
-      <c r="H17" s="11">
+      <c r="H17" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="F18" s="9" t="n"/>
       <c r="G18" s="9" t="n"/>
-      <c r="H18" s="11">
+      <c r="H18" s="10">
         <f>参数设置!$C$7</f>
         <v/>
       </c>
@@ -5770,7 +5770,7 @@
         <v/>
       </c>
       <c r="Q46" s="10">
-        <f>SUMPRODUCT((MOD(ROW(Q4:Q45)-4,14)=(12))*Q4:Q45)</f>
+        <f>SUMPRODUCT((MOD(ROW(Q4:Q45)-4,14)=(13))*Q4:Q45)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: upgrade warehouse template to 7-stage process flow
</commit_message>
<xml_diff>
--- a/manufacturing-warehouse-planning/仓库规划库存需求计算模板.xlsx
+++ b/manufacturing-warehouse-planning/仓库规划库存需求计算模板.xlsx
@@ -876,7 +876,7 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>BOM 表中需填写累计良率损耗系数（如工序1×工序2×工序3的综合良率倒数），以反映从原料到成品的实际消耗。</t>
+          <t>BOM 表中请填写单位成品实际原料消耗量（已包含粗破→烘干→磨粉→低温碳化→石墨化→高温碳化→成品筛分全流程良率损耗影响）。</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R14"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1339,7 +1339,11 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1436,24 +1440,52 @@
         <is>
           <t>过程品缓冲
 小时数
-(工序1后)</t>
+(粗破后)</t>
         </is>
       </c>
       <c r="P2" s="6" t="inlineStr">
         <is>
           <t>过程品缓冲
 小时数
-(工序2后)</t>
+(烘干后)</t>
         </is>
       </c>
       <c r="Q2" s="6" t="inlineStr">
         <is>
           <t>过程品缓冲
 小时数
-(工序3后)</t>
+(磨粉后)</t>
         </is>
       </c>
       <c r="R2" s="6" t="inlineStr">
+        <is>
+          <t>过程品缓冲
+小时数
+(低温碳化后)</t>
+        </is>
+      </c>
+      <c r="S2" s="6" t="inlineStr">
+        <is>
+          <t>过程品缓冲
+小时数
+(石墨化后)</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
+          <t>过程品缓冲
+小时数
+(高温碳化后)</t>
+        </is>
+      </c>
+      <c r="U2" s="6" t="inlineStr">
+        <is>
+          <t>过程品缓冲
+小时数
+(成品筛分后)</t>
+        </is>
+      </c>
+      <c r="V2" s="6" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -1511,15 +1543,27 @@
         <v>0.5</v>
       </c>
       <c r="O3" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P3" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q3" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="P3" s="11" t="n">
+      <c r="R3" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="S3" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="Q3" s="11" t="n">
+      <c r="T3" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="U3" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="R3" s="14" t="inlineStr"/>
+      <c r="V3" s="14" t="inlineStr"/>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="13" t="n">
@@ -1573,15 +1617,27 @@
         <v>0.6</v>
       </c>
       <c r="O4" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q4" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="P4" s="11" t="n">
+      <c r="R4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="S4" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="T4" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="Q4" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="R4" s="14" t="inlineStr"/>
+      <c r="U4" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="V4" s="14" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="13" t="n">
@@ -1638,12 +1694,24 @@
         <v>3</v>
       </c>
       <c r="P5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q5" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="Q5" s="11" t="n">
+      <c r="R5" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="S5" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T5" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="R5" s="14" t="inlineStr"/>
+      <c r="U5" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="V5" s="14" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="13" t="n">
@@ -1697,15 +1765,27 @@
         <v>0.4</v>
       </c>
       <c r="O6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="P6" s="11" t="n">
+      <c r="R6" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="S6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="Q6" s="11" t="n">
+      <c r="T6" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="U6" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="R6" s="14" t="inlineStr"/>
+      <c r="V6" s="14" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="13" t="n">
@@ -1759,15 +1839,27 @@
         <v>0.5</v>
       </c>
       <c r="O7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="P7" s="11" t="n">
+      <c r="Q7" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="Q7" s="11" t="n">
+      <c r="S7" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="T7" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="R7" s="14" t="inlineStr"/>
+      <c r="U7" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="V7" s="14" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="13" t="n">
@@ -1821,15 +1913,27 @@
         <v>0.7</v>
       </c>
       <c r="O8" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="R8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="P8" s="11" t="n">
+      <c r="S8" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="T8" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" s="14" t="inlineStr"/>
+      <c r="U8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="V8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="13" t="n">
@@ -1883,15 +1987,27 @@
         <v>1</v>
       </c>
       <c r="O9" s="11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P9" s="11" t="n">
         <v>5</v>
       </c>
       <c r="Q9" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="R9" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="R9" s="14" t="inlineStr"/>
+      <c r="S9" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="T9" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="U9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="V9" s="14" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="13" t="n">
@@ -1948,12 +2064,24 @@
         <v>3</v>
       </c>
       <c r="P10" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="Q10" s="11" t="n">
+      <c r="R10" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="S10" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="T10" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="R10" s="14" t="inlineStr"/>
+      <c r="U10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="V10" s="14" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" t="n">
@@ -1982,6 +2110,10 @@
       <c r="P11" s="14" t="n"/>
       <c r="Q11" s="14" t="n"/>
       <c r="R11" s="14" t="n"/>
+      <c r="S11" s="14" t="n"/>
+      <c r="T11" s="14" t="n"/>
+      <c r="U11" s="14" t="n"/>
+      <c r="V11" s="14" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" t="n">
@@ -2010,6 +2142,10 @@
       <c r="P12" s="14" t="n"/>
       <c r="Q12" s="14" t="n"/>
       <c r="R12" s="14" t="n"/>
+      <c r="S12" s="14" t="n"/>
+      <c r="T12" s="14" t="n"/>
+      <c r="U12" s="14" t="n"/>
+      <c r="V12" s="14" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" t="n">
@@ -2038,6 +2174,10 @@
       <c r="P13" s="14" t="n"/>
       <c r="Q13" s="14" t="n"/>
       <c r="R13" s="14" t="n"/>
+      <c r="S13" s="14" t="n"/>
+      <c r="T13" s="14" t="n"/>
+      <c r="U13" s="14" t="n"/>
+      <c r="V13" s="14" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" t="n">
@@ -2066,10 +2206,14 @@
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="14" t="n"/>
       <c r="R14" s="14" t="n"/>
+      <c r="S14" s="14" t="n"/>
+      <c r="T14" s="14" t="n"/>
+      <c r="U14" s="14" t="n"/>
+      <c r="V14" s="14" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3501,7 +3645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3644,7 +3788,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>【工序1后暂存】</t>
+          <t>【粗破后暂存】</t>
         </is>
       </c>
     </row>
@@ -3654,7 +3798,7 @@
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C5" s="16">
@@ -3711,7 +3855,7 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C6" s="16">
@@ -3768,7 +3912,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C7" s="16">
@@ -3825,7 +3969,7 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C8" s="16">
@@ -3882,7 +4026,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C9" s="16">
@@ -3939,7 +4083,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C10" s="16">
@@ -3996,7 +4140,7 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C11" s="16">
@@ -4053,7 +4197,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C12" s="16">
@@ -4110,7 +4254,7 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C13" s="16">
@@ -4167,7 +4311,7 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C14" s="16">
@@ -4224,7 +4368,7 @@
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C15" s="16">
@@ -4281,7 +4425,7 @@
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>工序1后暂存</t>
+          <t>粗破后暂存</t>
         </is>
       </c>
       <c r="C16" s="16">
@@ -4335,7 +4479,7 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
         <is>
-          <t>工序1后暂存 小计</t>
+          <t>粗破后暂存 小计</t>
         </is>
       </c>
       <c r="P17" s="10">
@@ -4350,7 +4494,7 @@
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>【工序2后暂存】</t>
+          <t>【烘干后暂存】</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4504,7 @@
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C19" s="16">
@@ -4417,7 +4561,7 @@
       </c>
       <c r="B20" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C20" s="16">
@@ -4474,7 +4618,7 @@
       </c>
       <c r="B21" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C21" s="16">
@@ -4531,7 +4675,7 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C22" s="16">
@@ -4588,7 +4732,7 @@
       </c>
       <c r="B23" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C23" s="16">
@@ -4645,7 +4789,7 @@
       </c>
       <c r="B24" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C24" s="16">
@@ -4702,7 +4846,7 @@
       </c>
       <c r="B25" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C25" s="16">
@@ -4759,7 +4903,7 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C26" s="16">
@@ -4816,7 +4960,7 @@
       </c>
       <c r="B27" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C27" s="16">
@@ -4873,7 +5017,7 @@
       </c>
       <c r="B28" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C28" s="16">
@@ -4930,7 +5074,7 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C29" s="16">
@@ -4987,7 +5131,7 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>工序2后暂存</t>
+          <t>烘干后暂存</t>
         </is>
       </c>
       <c r="C30" s="16">
@@ -5041,7 +5185,7 @@
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>工序2后暂存 小计</t>
+          <t>烘干后暂存 小计</t>
         </is>
       </c>
       <c r="P31" s="10">
@@ -5056,7 +5200,7 @@
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>【工序3后暂存（成品前）】</t>
+          <t>【磨粉后暂存】</t>
         </is>
       </c>
     </row>
@@ -5066,7 +5210,7 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C33" s="16">
@@ -5123,7 +5267,7 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C34" s="16">
@@ -5180,7 +5324,7 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C35" s="16">
@@ -5237,7 +5381,7 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C36" s="16">
@@ -5294,7 +5438,7 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C37" s="16">
@@ -5351,7 +5495,7 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C38" s="16">
@@ -5408,7 +5552,7 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C39" s="16">
@@ -5465,7 +5609,7 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C40" s="16">
@@ -5522,7 +5666,7 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C41" s="16">
@@ -5579,7 +5723,7 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C42" s="16">
@@ -5636,7 +5780,7 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C43" s="16">
@@ -5693,7 +5837,7 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前）</t>
+          <t>磨粉后暂存</t>
         </is>
       </c>
       <c r="C44" s="16">
@@ -5747,7 +5891,7 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
         <is>
-          <t>工序3后暂存（成品前） 小计</t>
+          <t>磨粉后暂存 小计</t>
         </is>
       </c>
       <c r="P45" s="10">
@@ -5760,30 +5904,2862 @@
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="18" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>【低温碳化后暂存】</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C47" s="16">
+        <f>IFERROR(产品SKU!B3,"")</f>
+        <v/>
+      </c>
+      <c r="D47" s="16">
+        <f>IFERROR(产品SKU!D3,"")</f>
+        <v/>
+      </c>
+      <c r="E47" s="10">
+        <f>IFERROR(产品SKU!G3,0)</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>IFERROR(过程品仓计算!E47/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G47" s="10">
+        <f>IFERROR(产品SKU!R3,0)</f>
+        <v/>
+      </c>
+      <c r="H47" s="10">
+        <f>IFERROR(过程品仓计算!F47*过程品仓计算!G47,0)</f>
+        <v/>
+      </c>
+      <c r="I47" s="9" t="n"/>
+      <c r="J47" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" s="10">
+        <f>IFERROR(IF(过程品仓计算!I47="",0,过程品仓计算!I47)*IF(过程品仓计算!J47="",0,过程品仓计算!J47),0)</f>
+        <v/>
+      </c>
+      <c r="L47" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H47,过程品仓计算!K47),0)</f>
+        <v/>
+      </c>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="9" t="n"/>
+      <c r="O47" s="9" t="n"/>
+      <c r="P47" s="10">
+        <f>IFERROR(过程品仓计算!L47+IF(过程品仓计算!M47="",0,过程品仓计算!M47)+IF(过程品仓计算!N47="",0,过程品仓计算!N47)+IF(过程品仓计算!O47="",0,过程品仓计算!O47),0)</f>
+        <v/>
+      </c>
+      <c r="Q47" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P47/MAX(产品SKU!M3,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C48" s="16">
+        <f>IFERROR(产品SKU!B4,"")</f>
+        <v/>
+      </c>
+      <c r="D48" s="16">
+        <f>IFERROR(产品SKU!D4,"")</f>
+        <v/>
+      </c>
+      <c r="E48" s="10">
+        <f>IFERROR(产品SKU!G4,0)</f>
+        <v/>
+      </c>
+      <c r="F48" s="10">
+        <f>IFERROR(过程品仓计算!E48/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G48" s="10">
+        <f>IFERROR(产品SKU!R4,0)</f>
+        <v/>
+      </c>
+      <c r="H48" s="10">
+        <f>IFERROR(过程品仓计算!F48*过程品仓计算!G48,0)</f>
+        <v/>
+      </c>
+      <c r="I48" s="9" t="n"/>
+      <c r="J48" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="10">
+        <f>IFERROR(IF(过程品仓计算!I48="",0,过程品仓计算!I48)*IF(过程品仓计算!J48="",0,过程品仓计算!J48),0)</f>
+        <v/>
+      </c>
+      <c r="L48" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H48,过程品仓计算!K48),0)</f>
+        <v/>
+      </c>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="9" t="n"/>
+      <c r="O48" s="9" t="n"/>
+      <c r="P48" s="10">
+        <f>IFERROR(过程品仓计算!L48+IF(过程品仓计算!M48="",0,过程品仓计算!M48)+IF(过程品仓计算!N48="",0,过程品仓计算!N48)+IF(过程品仓计算!O48="",0,过程品仓计算!O48),0)</f>
+        <v/>
+      </c>
+      <c r="Q48" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P48/MAX(产品SKU!M4,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C49" s="16">
+        <f>IFERROR(产品SKU!B5,"")</f>
+        <v/>
+      </c>
+      <c r="D49" s="16">
+        <f>IFERROR(产品SKU!D5,"")</f>
+        <v/>
+      </c>
+      <c r="E49" s="10">
+        <f>IFERROR(产品SKU!G5,0)</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>IFERROR(过程品仓计算!E49/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G49" s="10">
+        <f>IFERROR(产品SKU!R5,0)</f>
+        <v/>
+      </c>
+      <c r="H49" s="10">
+        <f>IFERROR(过程品仓计算!F49*过程品仓计算!G49,0)</f>
+        <v/>
+      </c>
+      <c r="I49" s="9" t="n"/>
+      <c r="J49" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K49" s="10">
+        <f>IFERROR(IF(过程品仓计算!I49="",0,过程品仓计算!I49)*IF(过程品仓计算!J49="",0,过程品仓计算!J49),0)</f>
+        <v/>
+      </c>
+      <c r="L49" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H49,过程品仓计算!K49),0)</f>
+        <v/>
+      </c>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="9" t="n"/>
+      <c r="O49" s="9" t="n"/>
+      <c r="P49" s="10">
+        <f>IFERROR(过程品仓计算!L49+IF(过程品仓计算!M49="",0,过程品仓计算!M49)+IF(过程品仓计算!N49="",0,过程品仓计算!N49)+IF(过程品仓计算!O49="",0,过程品仓计算!O49),0)</f>
+        <v/>
+      </c>
+      <c r="Q49" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P49/MAX(产品SKU!M5,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C50" s="16">
+        <f>IFERROR(产品SKU!B6,"")</f>
+        <v/>
+      </c>
+      <c r="D50" s="16">
+        <f>IFERROR(产品SKU!D6,"")</f>
+        <v/>
+      </c>
+      <c r="E50" s="10">
+        <f>IFERROR(产品SKU!G6,0)</f>
+        <v/>
+      </c>
+      <c r="F50" s="10">
+        <f>IFERROR(过程品仓计算!E50/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G50" s="10">
+        <f>IFERROR(产品SKU!R6,0)</f>
+        <v/>
+      </c>
+      <c r="H50" s="10">
+        <f>IFERROR(过程品仓计算!F50*过程品仓计算!G50,0)</f>
+        <v/>
+      </c>
+      <c r="I50" s="9" t="n"/>
+      <c r="J50" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K50" s="10">
+        <f>IFERROR(IF(过程品仓计算!I50="",0,过程品仓计算!I50)*IF(过程品仓计算!J50="",0,过程品仓计算!J50),0)</f>
+        <v/>
+      </c>
+      <c r="L50" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H50,过程品仓计算!K50),0)</f>
+        <v/>
+      </c>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+      <c r="O50" s="9" t="n"/>
+      <c r="P50" s="10">
+        <f>IFERROR(过程品仓计算!L50+IF(过程品仓计算!M50="",0,过程品仓计算!M50)+IF(过程品仓计算!N50="",0,过程品仓计算!N50)+IF(过程品仓计算!O50="",0,过程品仓计算!O50),0)</f>
+        <v/>
+      </c>
+      <c r="Q50" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P50/MAX(产品SKU!M6,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C51" s="16">
+        <f>IFERROR(产品SKU!B7,"")</f>
+        <v/>
+      </c>
+      <c r="D51" s="16">
+        <f>IFERROR(产品SKU!D7,"")</f>
+        <v/>
+      </c>
+      <c r="E51" s="10">
+        <f>IFERROR(产品SKU!G7,0)</f>
+        <v/>
+      </c>
+      <c r="F51" s="10">
+        <f>IFERROR(过程品仓计算!E51/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G51" s="10">
+        <f>IFERROR(产品SKU!R7,0)</f>
+        <v/>
+      </c>
+      <c r="H51" s="10">
+        <f>IFERROR(过程品仓计算!F51*过程品仓计算!G51,0)</f>
+        <v/>
+      </c>
+      <c r="I51" s="9" t="n"/>
+      <c r="J51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="10">
+        <f>IFERROR(IF(过程品仓计算!I51="",0,过程品仓计算!I51)*IF(过程品仓计算!J51="",0,过程品仓计算!J51),0)</f>
+        <v/>
+      </c>
+      <c r="L51" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H51,过程品仓计算!K51),0)</f>
+        <v/>
+      </c>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="9" t="n"/>
+      <c r="O51" s="9" t="n"/>
+      <c r="P51" s="10">
+        <f>IFERROR(过程品仓计算!L51+IF(过程品仓计算!M51="",0,过程品仓计算!M51)+IF(过程品仓计算!N51="",0,过程品仓计算!N51)+IF(过程品仓计算!O51="",0,过程品仓计算!O51),0)</f>
+        <v/>
+      </c>
+      <c r="Q51" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P51/MAX(产品SKU!M7,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C52" s="16">
+        <f>IFERROR(产品SKU!B8,"")</f>
+        <v/>
+      </c>
+      <c r="D52" s="16">
+        <f>IFERROR(产品SKU!D8,"")</f>
+        <v/>
+      </c>
+      <c r="E52" s="10">
+        <f>IFERROR(产品SKU!G8,0)</f>
+        <v/>
+      </c>
+      <c r="F52" s="10">
+        <f>IFERROR(过程品仓计算!E52/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G52" s="10">
+        <f>IFERROR(产品SKU!R8,0)</f>
+        <v/>
+      </c>
+      <c r="H52" s="10">
+        <f>IFERROR(过程品仓计算!F52*过程品仓计算!G52,0)</f>
+        <v/>
+      </c>
+      <c r="I52" s="9" t="n"/>
+      <c r="J52" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K52" s="10">
+        <f>IFERROR(IF(过程品仓计算!I52="",0,过程品仓计算!I52)*IF(过程品仓计算!J52="",0,过程品仓计算!J52),0)</f>
+        <v/>
+      </c>
+      <c r="L52" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H52,过程品仓计算!K52),0)</f>
+        <v/>
+      </c>
+      <c r="M52" s="9" t="n"/>
+      <c r="N52" s="9" t="n"/>
+      <c r="O52" s="9" t="n"/>
+      <c r="P52" s="10">
+        <f>IFERROR(过程品仓计算!L52+IF(过程品仓计算!M52="",0,过程品仓计算!M52)+IF(过程品仓计算!N52="",0,过程品仓计算!N52)+IF(过程品仓计算!O52="",0,过程品仓计算!O52),0)</f>
+        <v/>
+      </c>
+      <c r="Q52" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P52/MAX(产品SKU!M8,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C53" s="16">
+        <f>IFERROR(产品SKU!B9,"")</f>
+        <v/>
+      </c>
+      <c r="D53" s="16">
+        <f>IFERROR(产品SKU!D9,"")</f>
+        <v/>
+      </c>
+      <c r="E53" s="10">
+        <f>IFERROR(产品SKU!G9,0)</f>
+        <v/>
+      </c>
+      <c r="F53" s="10">
+        <f>IFERROR(过程品仓计算!E53/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G53" s="10">
+        <f>IFERROR(产品SKU!R9,0)</f>
+        <v/>
+      </c>
+      <c r="H53" s="10">
+        <f>IFERROR(过程品仓计算!F53*过程品仓计算!G53,0)</f>
+        <v/>
+      </c>
+      <c r="I53" s="9" t="n"/>
+      <c r="J53" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K53" s="10">
+        <f>IFERROR(IF(过程品仓计算!I53="",0,过程品仓计算!I53)*IF(过程品仓计算!J53="",0,过程品仓计算!J53),0)</f>
+        <v/>
+      </c>
+      <c r="L53" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H53,过程品仓计算!K53),0)</f>
+        <v/>
+      </c>
+      <c r="M53" s="9" t="n"/>
+      <c r="N53" s="9" t="n"/>
+      <c r="O53" s="9" t="n"/>
+      <c r="P53" s="10">
+        <f>IFERROR(过程品仓计算!L53+IF(过程品仓计算!M53="",0,过程品仓计算!M53)+IF(过程品仓计算!N53="",0,过程品仓计算!N53)+IF(过程品仓计算!O53="",0,过程品仓计算!O53),0)</f>
+        <v/>
+      </c>
+      <c r="Q53" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P53/MAX(产品SKU!M9,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C54" s="16">
+        <f>IFERROR(产品SKU!B10,"")</f>
+        <v/>
+      </c>
+      <c r="D54" s="16">
+        <f>IFERROR(产品SKU!D10,"")</f>
+        <v/>
+      </c>
+      <c r="E54" s="10">
+        <f>IFERROR(产品SKU!G10,0)</f>
+        <v/>
+      </c>
+      <c r="F54" s="10">
+        <f>IFERROR(过程品仓计算!E54/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G54" s="10">
+        <f>IFERROR(产品SKU!R10,0)</f>
+        <v/>
+      </c>
+      <c r="H54" s="10">
+        <f>IFERROR(过程品仓计算!F54*过程品仓计算!G54,0)</f>
+        <v/>
+      </c>
+      <c r="I54" s="9" t="n"/>
+      <c r="J54" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K54" s="10">
+        <f>IFERROR(IF(过程品仓计算!I54="",0,过程品仓计算!I54)*IF(过程品仓计算!J54="",0,过程品仓计算!J54),0)</f>
+        <v/>
+      </c>
+      <c r="L54" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H54,过程品仓计算!K54),0)</f>
+        <v/>
+      </c>
+      <c r="M54" s="9" t="n"/>
+      <c r="N54" s="9" t="n"/>
+      <c r="O54" s="9" t="n"/>
+      <c r="P54" s="10">
+        <f>IFERROR(过程品仓计算!L54+IF(过程品仓计算!M54="",0,过程品仓计算!M54)+IF(过程品仓计算!N54="",0,过程品仓计算!N54)+IF(过程品仓计算!O54="",0,过程品仓计算!O54),0)</f>
+        <v/>
+      </c>
+      <c r="Q54" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P54/MAX(产品SKU!M10,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C55" s="16">
+        <f>IFERROR(产品SKU!B11,"")</f>
+        <v/>
+      </c>
+      <c r="D55" s="16">
+        <f>IFERROR(产品SKU!D11,"")</f>
+        <v/>
+      </c>
+      <c r="E55" s="10">
+        <f>IFERROR(产品SKU!G11,0)</f>
+        <v/>
+      </c>
+      <c r="F55" s="10">
+        <f>IFERROR(过程品仓计算!E55/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G55" s="10">
+        <f>IFERROR(产品SKU!R11,0)</f>
+        <v/>
+      </c>
+      <c r="H55" s="10">
+        <f>IFERROR(过程品仓计算!F55*过程品仓计算!G55,0)</f>
+        <v/>
+      </c>
+      <c r="I55" s="9" t="n"/>
+      <c r="J55" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K55" s="10">
+        <f>IFERROR(IF(过程品仓计算!I55="",0,过程品仓计算!I55)*IF(过程品仓计算!J55="",0,过程品仓计算!J55),0)</f>
+        <v/>
+      </c>
+      <c r="L55" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H55,过程品仓计算!K55),0)</f>
+        <v/>
+      </c>
+      <c r="M55" s="9" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="10">
+        <f>IFERROR(过程品仓计算!L55+IF(过程品仓计算!M55="",0,过程品仓计算!M55)+IF(过程品仓计算!N55="",0,过程品仓计算!N55)+IF(过程品仓计算!O55="",0,过程品仓计算!O55),0)</f>
+        <v/>
+      </c>
+      <c r="Q55" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P55/MAX(产品SKU!M11,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="20" customHeight="1">
+      <c r="A56" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C56" s="16">
+        <f>IFERROR(产品SKU!B12,"")</f>
+        <v/>
+      </c>
+      <c r="D56" s="16">
+        <f>IFERROR(产品SKU!D12,"")</f>
+        <v/>
+      </c>
+      <c r="E56" s="10">
+        <f>IFERROR(产品SKU!G12,0)</f>
+        <v/>
+      </c>
+      <c r="F56" s="10">
+        <f>IFERROR(过程品仓计算!E56/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G56" s="10">
+        <f>IFERROR(产品SKU!R12,0)</f>
+        <v/>
+      </c>
+      <c r="H56" s="10">
+        <f>IFERROR(过程品仓计算!F56*过程品仓计算!G56,0)</f>
+        <v/>
+      </c>
+      <c r="I56" s="9" t="n"/>
+      <c r="J56" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="10">
+        <f>IFERROR(IF(过程品仓计算!I56="",0,过程品仓计算!I56)*IF(过程品仓计算!J56="",0,过程品仓计算!J56),0)</f>
+        <v/>
+      </c>
+      <c r="L56" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H56,过程品仓计算!K56),0)</f>
+        <v/>
+      </c>
+      <c r="M56" s="9" t="n"/>
+      <c r="N56" s="9" t="n"/>
+      <c r="O56" s="9" t="n"/>
+      <c r="P56" s="10">
+        <f>IFERROR(过程品仓计算!L56+IF(过程品仓计算!M56="",0,过程品仓计算!M56)+IF(过程品仓计算!N56="",0,过程品仓计算!N56)+IF(过程品仓计算!O56="",0,过程品仓计算!O56),0)</f>
+        <v/>
+      </c>
+      <c r="Q56" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P56/MAX(产品SKU!M12,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="20" customHeight="1">
+      <c r="A57" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C57" s="16">
+        <f>IFERROR(产品SKU!B13,"")</f>
+        <v/>
+      </c>
+      <c r="D57" s="16">
+        <f>IFERROR(产品SKU!D13,"")</f>
+        <v/>
+      </c>
+      <c r="E57" s="10">
+        <f>IFERROR(产品SKU!G13,0)</f>
+        <v/>
+      </c>
+      <c r="F57" s="10">
+        <f>IFERROR(过程品仓计算!E57/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G57" s="10">
+        <f>IFERROR(产品SKU!R13,0)</f>
+        <v/>
+      </c>
+      <c r="H57" s="10">
+        <f>IFERROR(过程品仓计算!F57*过程品仓计算!G57,0)</f>
+        <v/>
+      </c>
+      <c r="I57" s="9" t="n"/>
+      <c r="J57" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K57" s="10">
+        <f>IFERROR(IF(过程品仓计算!I57="",0,过程品仓计算!I57)*IF(过程品仓计算!J57="",0,过程品仓计算!J57),0)</f>
+        <v/>
+      </c>
+      <c r="L57" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H57,过程品仓计算!K57),0)</f>
+        <v/>
+      </c>
+      <c r="M57" s="9" t="n"/>
+      <c r="N57" s="9" t="n"/>
+      <c r="O57" s="9" t="n"/>
+      <c r="P57" s="10">
+        <f>IFERROR(过程品仓计算!L57+IF(过程品仓计算!M57="",0,过程品仓计算!M57)+IF(过程品仓计算!N57="",0,过程品仓计算!N57)+IF(过程品仓计算!O57="",0,过程品仓计算!O57),0)</f>
+        <v/>
+      </c>
+      <c r="Q57" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P57/MAX(产品SKU!M13,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="20" customHeight="1">
+      <c r="A58" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C58" s="16">
+        <f>IFERROR(产品SKU!B14,"")</f>
+        <v/>
+      </c>
+      <c r="D58" s="16">
+        <f>IFERROR(产品SKU!D14,"")</f>
+        <v/>
+      </c>
+      <c r="E58" s="10">
+        <f>IFERROR(产品SKU!G14,0)</f>
+        <v/>
+      </c>
+      <c r="F58" s="10">
+        <f>IFERROR(过程品仓计算!E58/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G58" s="10">
+        <f>IFERROR(产品SKU!R14,0)</f>
+        <v/>
+      </c>
+      <c r="H58" s="10">
+        <f>IFERROR(过程品仓计算!F58*过程品仓计算!G58,0)</f>
+        <v/>
+      </c>
+      <c r="I58" s="9" t="n"/>
+      <c r="J58" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K58" s="10">
+        <f>IFERROR(IF(过程品仓计算!I58="",0,过程品仓计算!I58)*IF(过程品仓计算!J58="",0,过程品仓计算!J58),0)</f>
+        <v/>
+      </c>
+      <c r="L58" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H58,过程品仓计算!K58),0)</f>
+        <v/>
+      </c>
+      <c r="M58" s="9" t="n"/>
+      <c r="N58" s="9" t="n"/>
+      <c r="O58" s="9" t="n"/>
+      <c r="P58" s="10">
+        <f>IFERROR(过程品仓计算!L58+IF(过程品仓计算!M58="",0,过程品仓计算!M58)+IF(过程品仓计算!N58="",0,过程品仓计算!N58)+IF(过程品仓计算!O58="",0,过程品仓计算!O58),0)</f>
+        <v/>
+      </c>
+      <c r="Q58" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P58/MAX(产品SKU!M14,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="20" customHeight="1">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>低温碳化后暂存 小计</t>
+        </is>
+      </c>
+      <c r="P59" s="10">
+        <f>SUM(P47:P58)</f>
+        <v/>
+      </c>
+      <c r="Q59" s="10">
+        <f>SUM(Q47:Q58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>【石墨化后暂存】</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C61" s="16">
+        <f>IFERROR(产品SKU!B3,"")</f>
+        <v/>
+      </c>
+      <c r="D61" s="16">
+        <f>IFERROR(产品SKU!D3,"")</f>
+        <v/>
+      </c>
+      <c r="E61" s="10">
+        <f>IFERROR(产品SKU!G3,0)</f>
+        <v/>
+      </c>
+      <c r="F61" s="10">
+        <f>IFERROR(过程品仓计算!E61/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G61" s="10">
+        <f>IFERROR(产品SKU!S3,0)</f>
+        <v/>
+      </c>
+      <c r="H61" s="10">
+        <f>IFERROR(过程品仓计算!F61*过程品仓计算!G61,0)</f>
+        <v/>
+      </c>
+      <c r="I61" s="9" t="n"/>
+      <c r="J61" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K61" s="10">
+        <f>IFERROR(IF(过程品仓计算!I61="",0,过程品仓计算!I61)*IF(过程品仓计算!J61="",0,过程品仓计算!J61),0)</f>
+        <v/>
+      </c>
+      <c r="L61" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H61,过程品仓计算!K61),0)</f>
+        <v/>
+      </c>
+      <c r="M61" s="9" t="n"/>
+      <c r="N61" s="9" t="n"/>
+      <c r="O61" s="9" t="n"/>
+      <c r="P61" s="10">
+        <f>IFERROR(过程品仓计算!L61+IF(过程品仓计算!M61="",0,过程品仓计算!M61)+IF(过程品仓计算!N61="",0,过程品仓计算!N61)+IF(过程品仓计算!O61="",0,过程品仓计算!O61),0)</f>
+        <v/>
+      </c>
+      <c r="Q61" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P61/MAX(产品SKU!M3,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C62" s="16">
+        <f>IFERROR(产品SKU!B4,"")</f>
+        <v/>
+      </c>
+      <c r="D62" s="16">
+        <f>IFERROR(产品SKU!D4,"")</f>
+        <v/>
+      </c>
+      <c r="E62" s="10">
+        <f>IFERROR(产品SKU!G4,0)</f>
+        <v/>
+      </c>
+      <c r="F62" s="10">
+        <f>IFERROR(过程品仓计算!E62/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G62" s="10">
+        <f>IFERROR(产品SKU!S4,0)</f>
+        <v/>
+      </c>
+      <c r="H62" s="10">
+        <f>IFERROR(过程品仓计算!F62*过程品仓计算!G62,0)</f>
+        <v/>
+      </c>
+      <c r="I62" s="9" t="n"/>
+      <c r="J62" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K62" s="10">
+        <f>IFERROR(IF(过程品仓计算!I62="",0,过程品仓计算!I62)*IF(过程品仓计算!J62="",0,过程品仓计算!J62),0)</f>
+        <v/>
+      </c>
+      <c r="L62" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H62,过程品仓计算!K62),0)</f>
+        <v/>
+      </c>
+      <c r="M62" s="9" t="n"/>
+      <c r="N62" s="9" t="n"/>
+      <c r="O62" s="9" t="n"/>
+      <c r="P62" s="10">
+        <f>IFERROR(过程品仓计算!L62+IF(过程品仓计算!M62="",0,过程品仓计算!M62)+IF(过程品仓计算!N62="",0,过程品仓计算!N62)+IF(过程品仓计算!O62="",0,过程品仓计算!O62),0)</f>
+        <v/>
+      </c>
+      <c r="Q62" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P62/MAX(产品SKU!M4,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="20" customHeight="1">
+      <c r="A63" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C63" s="16">
+        <f>IFERROR(产品SKU!B5,"")</f>
+        <v/>
+      </c>
+      <c r="D63" s="16">
+        <f>IFERROR(产品SKU!D5,"")</f>
+        <v/>
+      </c>
+      <c r="E63" s="10">
+        <f>IFERROR(产品SKU!G5,0)</f>
+        <v/>
+      </c>
+      <c r="F63" s="10">
+        <f>IFERROR(过程品仓计算!E63/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G63" s="10">
+        <f>IFERROR(产品SKU!S5,0)</f>
+        <v/>
+      </c>
+      <c r="H63" s="10">
+        <f>IFERROR(过程品仓计算!F63*过程品仓计算!G63,0)</f>
+        <v/>
+      </c>
+      <c r="I63" s="9" t="n"/>
+      <c r="J63" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K63" s="10">
+        <f>IFERROR(IF(过程品仓计算!I63="",0,过程品仓计算!I63)*IF(过程品仓计算!J63="",0,过程品仓计算!J63),0)</f>
+        <v/>
+      </c>
+      <c r="L63" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H63,过程品仓计算!K63),0)</f>
+        <v/>
+      </c>
+      <c r="M63" s="9" t="n"/>
+      <c r="N63" s="9" t="n"/>
+      <c r="O63" s="9" t="n"/>
+      <c r="P63" s="10">
+        <f>IFERROR(过程品仓计算!L63+IF(过程品仓计算!M63="",0,过程品仓计算!M63)+IF(过程品仓计算!N63="",0,过程品仓计算!N63)+IF(过程品仓计算!O63="",0,过程品仓计算!O63),0)</f>
+        <v/>
+      </c>
+      <c r="Q63" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P63/MAX(产品SKU!M5,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="20" customHeight="1">
+      <c r="A64" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C64" s="16">
+        <f>IFERROR(产品SKU!B6,"")</f>
+        <v/>
+      </c>
+      <c r="D64" s="16">
+        <f>IFERROR(产品SKU!D6,"")</f>
+        <v/>
+      </c>
+      <c r="E64" s="10">
+        <f>IFERROR(产品SKU!G6,0)</f>
+        <v/>
+      </c>
+      <c r="F64" s="10">
+        <f>IFERROR(过程品仓计算!E64/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G64" s="10">
+        <f>IFERROR(产品SKU!S6,0)</f>
+        <v/>
+      </c>
+      <c r="H64" s="10">
+        <f>IFERROR(过程品仓计算!F64*过程品仓计算!G64,0)</f>
+        <v/>
+      </c>
+      <c r="I64" s="9" t="n"/>
+      <c r="J64" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K64" s="10">
+        <f>IFERROR(IF(过程品仓计算!I64="",0,过程品仓计算!I64)*IF(过程品仓计算!J64="",0,过程品仓计算!J64),0)</f>
+        <v/>
+      </c>
+      <c r="L64" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H64,过程品仓计算!K64),0)</f>
+        <v/>
+      </c>
+      <c r="M64" s="9" t="n"/>
+      <c r="N64" s="9" t="n"/>
+      <c r="O64" s="9" t="n"/>
+      <c r="P64" s="10">
+        <f>IFERROR(过程品仓计算!L64+IF(过程品仓计算!M64="",0,过程品仓计算!M64)+IF(过程品仓计算!N64="",0,过程品仓计算!N64)+IF(过程品仓计算!O64="",0,过程品仓计算!O64),0)</f>
+        <v/>
+      </c>
+      <c r="Q64" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P64/MAX(产品SKU!M6,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="A65" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C65" s="16">
+        <f>IFERROR(产品SKU!B7,"")</f>
+        <v/>
+      </c>
+      <c r="D65" s="16">
+        <f>IFERROR(产品SKU!D7,"")</f>
+        <v/>
+      </c>
+      <c r="E65" s="10">
+        <f>IFERROR(产品SKU!G7,0)</f>
+        <v/>
+      </c>
+      <c r="F65" s="10">
+        <f>IFERROR(过程品仓计算!E65/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G65" s="10">
+        <f>IFERROR(产品SKU!S7,0)</f>
+        <v/>
+      </c>
+      <c r="H65" s="10">
+        <f>IFERROR(过程品仓计算!F65*过程品仓计算!G65,0)</f>
+        <v/>
+      </c>
+      <c r="I65" s="9" t="n"/>
+      <c r="J65" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K65" s="10">
+        <f>IFERROR(IF(过程品仓计算!I65="",0,过程品仓计算!I65)*IF(过程品仓计算!J65="",0,过程品仓计算!J65),0)</f>
+        <v/>
+      </c>
+      <c r="L65" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H65,过程品仓计算!K65),0)</f>
+        <v/>
+      </c>
+      <c r="M65" s="9" t="n"/>
+      <c r="N65" s="9" t="n"/>
+      <c r="O65" s="9" t="n"/>
+      <c r="P65" s="10">
+        <f>IFERROR(过程品仓计算!L65+IF(过程品仓计算!M65="",0,过程品仓计算!M65)+IF(过程品仓计算!N65="",0,过程品仓计算!N65)+IF(过程品仓计算!O65="",0,过程品仓计算!O65),0)</f>
+        <v/>
+      </c>
+      <c r="Q65" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P65/MAX(产品SKU!M7,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="20" customHeight="1">
+      <c r="A66" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C66" s="16">
+        <f>IFERROR(产品SKU!B8,"")</f>
+        <v/>
+      </c>
+      <c r="D66" s="16">
+        <f>IFERROR(产品SKU!D8,"")</f>
+        <v/>
+      </c>
+      <c r="E66" s="10">
+        <f>IFERROR(产品SKU!G8,0)</f>
+        <v/>
+      </c>
+      <c r="F66" s="10">
+        <f>IFERROR(过程品仓计算!E66/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G66" s="10">
+        <f>IFERROR(产品SKU!S8,0)</f>
+        <v/>
+      </c>
+      <c r="H66" s="10">
+        <f>IFERROR(过程品仓计算!F66*过程品仓计算!G66,0)</f>
+        <v/>
+      </c>
+      <c r="I66" s="9" t="n"/>
+      <c r="J66" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K66" s="10">
+        <f>IFERROR(IF(过程品仓计算!I66="",0,过程品仓计算!I66)*IF(过程品仓计算!J66="",0,过程品仓计算!J66),0)</f>
+        <v/>
+      </c>
+      <c r="L66" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H66,过程品仓计算!K66),0)</f>
+        <v/>
+      </c>
+      <c r="M66" s="9" t="n"/>
+      <c r="N66" s="9" t="n"/>
+      <c r="O66" s="9" t="n"/>
+      <c r="P66" s="10">
+        <f>IFERROR(过程品仓计算!L66+IF(过程品仓计算!M66="",0,过程品仓计算!M66)+IF(过程品仓计算!N66="",0,过程品仓计算!N66)+IF(过程品仓计算!O66="",0,过程品仓计算!O66),0)</f>
+        <v/>
+      </c>
+      <c r="Q66" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P66/MAX(产品SKU!M8,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="20" customHeight="1">
+      <c r="A67" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C67" s="16">
+        <f>IFERROR(产品SKU!B9,"")</f>
+        <v/>
+      </c>
+      <c r="D67" s="16">
+        <f>IFERROR(产品SKU!D9,"")</f>
+        <v/>
+      </c>
+      <c r="E67" s="10">
+        <f>IFERROR(产品SKU!G9,0)</f>
+        <v/>
+      </c>
+      <c r="F67" s="10">
+        <f>IFERROR(过程品仓计算!E67/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G67" s="10">
+        <f>IFERROR(产品SKU!S9,0)</f>
+        <v/>
+      </c>
+      <c r="H67" s="10">
+        <f>IFERROR(过程品仓计算!F67*过程品仓计算!G67,0)</f>
+        <v/>
+      </c>
+      <c r="I67" s="9" t="n"/>
+      <c r="J67" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K67" s="10">
+        <f>IFERROR(IF(过程品仓计算!I67="",0,过程品仓计算!I67)*IF(过程品仓计算!J67="",0,过程品仓计算!J67),0)</f>
+        <v/>
+      </c>
+      <c r="L67" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H67,过程品仓计算!K67),0)</f>
+        <v/>
+      </c>
+      <c r="M67" s="9" t="n"/>
+      <c r="N67" s="9" t="n"/>
+      <c r="O67" s="9" t="n"/>
+      <c r="P67" s="10">
+        <f>IFERROR(过程品仓计算!L67+IF(过程品仓计算!M67="",0,过程品仓计算!M67)+IF(过程品仓计算!N67="",0,过程品仓计算!N67)+IF(过程品仓计算!O67="",0,过程品仓计算!O67),0)</f>
+        <v/>
+      </c>
+      <c r="Q67" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P67/MAX(产品SKU!M9,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" ht="20" customHeight="1">
+      <c r="A68" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C68" s="16">
+        <f>IFERROR(产品SKU!B10,"")</f>
+        <v/>
+      </c>
+      <c r="D68" s="16">
+        <f>IFERROR(产品SKU!D10,"")</f>
+        <v/>
+      </c>
+      <c r="E68" s="10">
+        <f>IFERROR(产品SKU!G10,0)</f>
+        <v/>
+      </c>
+      <c r="F68" s="10">
+        <f>IFERROR(过程品仓计算!E68/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G68" s="10">
+        <f>IFERROR(产品SKU!S10,0)</f>
+        <v/>
+      </c>
+      <c r="H68" s="10">
+        <f>IFERROR(过程品仓计算!F68*过程品仓计算!G68,0)</f>
+        <v/>
+      </c>
+      <c r="I68" s="9" t="n"/>
+      <c r="J68" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K68" s="10">
+        <f>IFERROR(IF(过程品仓计算!I68="",0,过程品仓计算!I68)*IF(过程品仓计算!J68="",0,过程品仓计算!J68),0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H68,过程品仓计算!K68),0)</f>
+        <v/>
+      </c>
+      <c r="M68" s="9" t="n"/>
+      <c r="N68" s="9" t="n"/>
+      <c r="O68" s="9" t="n"/>
+      <c r="P68" s="10">
+        <f>IFERROR(过程品仓计算!L68+IF(过程品仓计算!M68="",0,过程品仓计算!M68)+IF(过程品仓计算!N68="",0,过程品仓计算!N68)+IF(过程品仓计算!O68="",0,过程品仓计算!O68),0)</f>
+        <v/>
+      </c>
+      <c r="Q68" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P68/MAX(产品SKU!M10,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="20" customHeight="1">
+      <c r="A69" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C69" s="16">
+        <f>IFERROR(产品SKU!B11,"")</f>
+        <v/>
+      </c>
+      <c r="D69" s="16">
+        <f>IFERROR(产品SKU!D11,"")</f>
+        <v/>
+      </c>
+      <c r="E69" s="10">
+        <f>IFERROR(产品SKU!G11,0)</f>
+        <v/>
+      </c>
+      <c r="F69" s="10">
+        <f>IFERROR(过程品仓计算!E69/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G69" s="10">
+        <f>IFERROR(产品SKU!S11,0)</f>
+        <v/>
+      </c>
+      <c r="H69" s="10">
+        <f>IFERROR(过程品仓计算!F69*过程品仓计算!G69,0)</f>
+        <v/>
+      </c>
+      <c r="I69" s="9" t="n"/>
+      <c r="J69" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K69" s="10">
+        <f>IFERROR(IF(过程品仓计算!I69="",0,过程品仓计算!I69)*IF(过程品仓计算!J69="",0,过程品仓计算!J69),0)</f>
+        <v/>
+      </c>
+      <c r="L69" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H69,过程品仓计算!K69),0)</f>
+        <v/>
+      </c>
+      <c r="M69" s="9" t="n"/>
+      <c r="N69" s="9" t="n"/>
+      <c r="O69" s="9" t="n"/>
+      <c r="P69" s="10">
+        <f>IFERROR(过程品仓计算!L69+IF(过程品仓计算!M69="",0,过程品仓计算!M69)+IF(过程品仓计算!N69="",0,过程品仓计算!N69)+IF(过程品仓计算!O69="",0,过程品仓计算!O69),0)</f>
+        <v/>
+      </c>
+      <c r="Q69" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P69/MAX(产品SKU!M11,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="A70" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C70" s="16">
+        <f>IFERROR(产品SKU!B12,"")</f>
+        <v/>
+      </c>
+      <c r="D70" s="16">
+        <f>IFERROR(产品SKU!D12,"")</f>
+        <v/>
+      </c>
+      <c r="E70" s="10">
+        <f>IFERROR(产品SKU!G12,0)</f>
+        <v/>
+      </c>
+      <c r="F70" s="10">
+        <f>IFERROR(过程品仓计算!E70/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G70" s="10">
+        <f>IFERROR(产品SKU!S12,0)</f>
+        <v/>
+      </c>
+      <c r="H70" s="10">
+        <f>IFERROR(过程品仓计算!F70*过程品仓计算!G70,0)</f>
+        <v/>
+      </c>
+      <c r="I70" s="9" t="n"/>
+      <c r="J70" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K70" s="10">
+        <f>IFERROR(IF(过程品仓计算!I70="",0,过程品仓计算!I70)*IF(过程品仓计算!J70="",0,过程品仓计算!J70),0)</f>
+        <v/>
+      </c>
+      <c r="L70" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H70,过程品仓计算!K70),0)</f>
+        <v/>
+      </c>
+      <c r="M70" s="9" t="n"/>
+      <c r="N70" s="9" t="n"/>
+      <c r="O70" s="9" t="n"/>
+      <c r="P70" s="10">
+        <f>IFERROR(过程品仓计算!L70+IF(过程品仓计算!M70="",0,过程品仓计算!M70)+IF(过程品仓计算!N70="",0,过程品仓计算!N70)+IF(过程品仓计算!O70="",0,过程品仓计算!O70),0)</f>
+        <v/>
+      </c>
+      <c r="Q70" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P70/MAX(产品SKU!M12,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="20" customHeight="1">
+      <c r="A71" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C71" s="16">
+        <f>IFERROR(产品SKU!B13,"")</f>
+        <v/>
+      </c>
+      <c r="D71" s="16">
+        <f>IFERROR(产品SKU!D13,"")</f>
+        <v/>
+      </c>
+      <c r="E71" s="10">
+        <f>IFERROR(产品SKU!G13,0)</f>
+        <v/>
+      </c>
+      <c r="F71" s="10">
+        <f>IFERROR(过程品仓计算!E71/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G71" s="10">
+        <f>IFERROR(产品SKU!S13,0)</f>
+        <v/>
+      </c>
+      <c r="H71" s="10">
+        <f>IFERROR(过程品仓计算!F71*过程品仓计算!G71,0)</f>
+        <v/>
+      </c>
+      <c r="I71" s="9" t="n"/>
+      <c r="J71" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K71" s="10">
+        <f>IFERROR(IF(过程品仓计算!I71="",0,过程品仓计算!I71)*IF(过程品仓计算!J71="",0,过程品仓计算!J71),0)</f>
+        <v/>
+      </c>
+      <c r="L71" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H71,过程品仓计算!K71),0)</f>
+        <v/>
+      </c>
+      <c r="M71" s="9" t="n"/>
+      <c r="N71" s="9" t="n"/>
+      <c r="O71" s="9" t="n"/>
+      <c r="P71" s="10">
+        <f>IFERROR(过程品仓计算!L71+IF(过程品仓计算!M71="",0,过程品仓计算!M71)+IF(过程品仓计算!N71="",0,过程品仓计算!N71)+IF(过程品仓计算!O71="",0,过程品仓计算!O71),0)</f>
+        <v/>
+      </c>
+      <c r="Q71" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P71/MAX(产品SKU!M13,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" ht="20" customHeight="1">
+      <c r="A72" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B72" s="16" t="inlineStr">
+        <is>
+          <t>石墨化后暂存</t>
+        </is>
+      </c>
+      <c r="C72" s="16">
+        <f>IFERROR(产品SKU!B14,"")</f>
+        <v/>
+      </c>
+      <c r="D72" s="16">
+        <f>IFERROR(产品SKU!D14,"")</f>
+        <v/>
+      </c>
+      <c r="E72" s="10">
+        <f>IFERROR(产品SKU!G14,0)</f>
+        <v/>
+      </c>
+      <c r="F72" s="10">
+        <f>IFERROR(过程品仓计算!E72/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G72" s="10">
+        <f>IFERROR(产品SKU!S14,0)</f>
+        <v/>
+      </c>
+      <c r="H72" s="10">
+        <f>IFERROR(过程品仓计算!F72*过程品仓计算!G72,0)</f>
+        <v/>
+      </c>
+      <c r="I72" s="9" t="n"/>
+      <c r="J72" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K72" s="10">
+        <f>IFERROR(IF(过程品仓计算!I72="",0,过程品仓计算!I72)*IF(过程品仓计算!J72="",0,过程品仓计算!J72),0)</f>
+        <v/>
+      </c>
+      <c r="L72" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H72,过程品仓计算!K72),0)</f>
+        <v/>
+      </c>
+      <c r="M72" s="9" t="n"/>
+      <c r="N72" s="9" t="n"/>
+      <c r="O72" s="9" t="n"/>
+      <c r="P72" s="10">
+        <f>IFERROR(过程品仓计算!L72+IF(过程品仓计算!M72="",0,过程品仓计算!M72)+IF(过程品仓计算!N72="",0,过程品仓计算!N72)+IF(过程品仓计算!O72="",0,过程品仓计算!O72),0)</f>
+        <v/>
+      </c>
+      <c r="Q72" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P72/MAX(产品SKU!M14,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="20" customHeight="1">
+      <c r="A73" s="19" t="inlineStr">
+        <is>
+          <t>石墨化后暂存 小计</t>
+        </is>
+      </c>
+      <c r="P73" s="10">
+        <f>SUM(P61:P72)</f>
+        <v/>
+      </c>
+      <c r="Q73" s="10">
+        <f>SUM(Q61:Q72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>【高温碳化后暂存】</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="20" customHeight="1">
+      <c r="A75" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C75" s="16">
+        <f>IFERROR(产品SKU!B3,"")</f>
+        <v/>
+      </c>
+      <c r="D75" s="16">
+        <f>IFERROR(产品SKU!D3,"")</f>
+        <v/>
+      </c>
+      <c r="E75" s="10">
+        <f>IFERROR(产品SKU!G3,0)</f>
+        <v/>
+      </c>
+      <c r="F75" s="10">
+        <f>IFERROR(过程品仓计算!E75/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G75" s="10">
+        <f>IFERROR(产品SKU!T3,0)</f>
+        <v/>
+      </c>
+      <c r="H75" s="10">
+        <f>IFERROR(过程品仓计算!F75*过程品仓计算!G75,0)</f>
+        <v/>
+      </c>
+      <c r="I75" s="9" t="n"/>
+      <c r="J75" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K75" s="10">
+        <f>IFERROR(IF(过程品仓计算!I75="",0,过程品仓计算!I75)*IF(过程品仓计算!J75="",0,过程品仓计算!J75),0)</f>
+        <v/>
+      </c>
+      <c r="L75" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H75,过程品仓计算!K75),0)</f>
+        <v/>
+      </c>
+      <c r="M75" s="9" t="n"/>
+      <c r="N75" s="9" t="n"/>
+      <c r="O75" s="9" t="n"/>
+      <c r="P75" s="10">
+        <f>IFERROR(过程品仓计算!L75+IF(过程品仓计算!M75="",0,过程品仓计算!M75)+IF(过程品仓计算!N75="",0,过程品仓计算!N75)+IF(过程品仓计算!O75="",0,过程品仓计算!O75),0)</f>
+        <v/>
+      </c>
+      <c r="Q75" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P75/MAX(产品SKU!M3,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="20" customHeight="1">
+      <c r="A76" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C76" s="16">
+        <f>IFERROR(产品SKU!B4,"")</f>
+        <v/>
+      </c>
+      <c r="D76" s="16">
+        <f>IFERROR(产品SKU!D4,"")</f>
+        <v/>
+      </c>
+      <c r="E76" s="10">
+        <f>IFERROR(产品SKU!G4,0)</f>
+        <v/>
+      </c>
+      <c r="F76" s="10">
+        <f>IFERROR(过程品仓计算!E76/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G76" s="10">
+        <f>IFERROR(产品SKU!T4,0)</f>
+        <v/>
+      </c>
+      <c r="H76" s="10">
+        <f>IFERROR(过程品仓计算!F76*过程品仓计算!G76,0)</f>
+        <v/>
+      </c>
+      <c r="I76" s="9" t="n"/>
+      <c r="J76" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K76" s="10">
+        <f>IFERROR(IF(过程品仓计算!I76="",0,过程品仓计算!I76)*IF(过程品仓计算!J76="",0,过程品仓计算!J76),0)</f>
+        <v/>
+      </c>
+      <c r="L76" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H76,过程品仓计算!K76),0)</f>
+        <v/>
+      </c>
+      <c r="M76" s="9" t="n"/>
+      <c r="N76" s="9" t="n"/>
+      <c r="O76" s="9" t="n"/>
+      <c r="P76" s="10">
+        <f>IFERROR(过程品仓计算!L76+IF(过程品仓计算!M76="",0,过程品仓计算!M76)+IF(过程品仓计算!N76="",0,过程品仓计算!N76)+IF(过程品仓计算!O76="",0,过程品仓计算!O76),0)</f>
+        <v/>
+      </c>
+      <c r="Q76" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P76/MAX(产品SKU!M4,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="20" customHeight="1">
+      <c r="A77" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C77" s="16">
+        <f>IFERROR(产品SKU!B5,"")</f>
+        <v/>
+      </c>
+      <c r="D77" s="16">
+        <f>IFERROR(产品SKU!D5,"")</f>
+        <v/>
+      </c>
+      <c r="E77" s="10">
+        <f>IFERROR(产品SKU!G5,0)</f>
+        <v/>
+      </c>
+      <c r="F77" s="10">
+        <f>IFERROR(过程品仓计算!E77/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G77" s="10">
+        <f>IFERROR(产品SKU!T5,0)</f>
+        <v/>
+      </c>
+      <c r="H77" s="10">
+        <f>IFERROR(过程品仓计算!F77*过程品仓计算!G77,0)</f>
+        <v/>
+      </c>
+      <c r="I77" s="9" t="n"/>
+      <c r="J77" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K77" s="10">
+        <f>IFERROR(IF(过程品仓计算!I77="",0,过程品仓计算!I77)*IF(过程品仓计算!J77="",0,过程品仓计算!J77),0)</f>
+        <v/>
+      </c>
+      <c r="L77" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H77,过程品仓计算!K77),0)</f>
+        <v/>
+      </c>
+      <c r="M77" s="9" t="n"/>
+      <c r="N77" s="9" t="n"/>
+      <c r="O77" s="9" t="n"/>
+      <c r="P77" s="10">
+        <f>IFERROR(过程品仓计算!L77+IF(过程品仓计算!M77="",0,过程品仓计算!M77)+IF(过程品仓计算!N77="",0,过程品仓计算!N77)+IF(过程品仓计算!O77="",0,过程品仓计算!O77),0)</f>
+        <v/>
+      </c>
+      <c r="Q77" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P77/MAX(产品SKU!M5,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="A78" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C78" s="16">
+        <f>IFERROR(产品SKU!B6,"")</f>
+        <v/>
+      </c>
+      <c r="D78" s="16">
+        <f>IFERROR(产品SKU!D6,"")</f>
+        <v/>
+      </c>
+      <c r="E78" s="10">
+        <f>IFERROR(产品SKU!G6,0)</f>
+        <v/>
+      </c>
+      <c r="F78" s="10">
+        <f>IFERROR(过程品仓计算!E78/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G78" s="10">
+        <f>IFERROR(产品SKU!T6,0)</f>
+        <v/>
+      </c>
+      <c r="H78" s="10">
+        <f>IFERROR(过程品仓计算!F78*过程品仓计算!G78,0)</f>
+        <v/>
+      </c>
+      <c r="I78" s="9" t="n"/>
+      <c r="J78" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K78" s="10">
+        <f>IFERROR(IF(过程品仓计算!I78="",0,过程品仓计算!I78)*IF(过程品仓计算!J78="",0,过程品仓计算!J78),0)</f>
+        <v/>
+      </c>
+      <c r="L78" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H78,过程品仓计算!K78),0)</f>
+        <v/>
+      </c>
+      <c r="M78" s="9" t="n"/>
+      <c r="N78" s="9" t="n"/>
+      <c r="O78" s="9" t="n"/>
+      <c r="P78" s="10">
+        <f>IFERROR(过程品仓计算!L78+IF(过程品仓计算!M78="",0,过程品仓计算!M78)+IF(过程品仓计算!N78="",0,过程品仓计算!N78)+IF(过程品仓计算!O78="",0,过程品仓计算!O78),0)</f>
+        <v/>
+      </c>
+      <c r="Q78" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P78/MAX(产品SKU!M6,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="20" customHeight="1">
+      <c r="A79" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C79" s="16">
+        <f>IFERROR(产品SKU!B7,"")</f>
+        <v/>
+      </c>
+      <c r="D79" s="16">
+        <f>IFERROR(产品SKU!D7,"")</f>
+        <v/>
+      </c>
+      <c r="E79" s="10">
+        <f>IFERROR(产品SKU!G7,0)</f>
+        <v/>
+      </c>
+      <c r="F79" s="10">
+        <f>IFERROR(过程品仓计算!E79/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G79" s="10">
+        <f>IFERROR(产品SKU!T7,0)</f>
+        <v/>
+      </c>
+      <c r="H79" s="10">
+        <f>IFERROR(过程品仓计算!F79*过程品仓计算!G79,0)</f>
+        <v/>
+      </c>
+      <c r="I79" s="9" t="n"/>
+      <c r="J79" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K79" s="10">
+        <f>IFERROR(IF(过程品仓计算!I79="",0,过程品仓计算!I79)*IF(过程品仓计算!J79="",0,过程品仓计算!J79),0)</f>
+        <v/>
+      </c>
+      <c r="L79" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H79,过程品仓计算!K79),0)</f>
+        <v/>
+      </c>
+      <c r="M79" s="9" t="n"/>
+      <c r="N79" s="9" t="n"/>
+      <c r="O79" s="9" t="n"/>
+      <c r="P79" s="10">
+        <f>IFERROR(过程品仓计算!L79+IF(过程品仓计算!M79="",0,过程品仓计算!M79)+IF(过程品仓计算!N79="",0,过程品仓计算!N79)+IF(过程品仓计算!O79="",0,过程品仓计算!O79),0)</f>
+        <v/>
+      </c>
+      <c r="Q79" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P79/MAX(产品SKU!M7,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" ht="20" customHeight="1">
+      <c r="A80" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C80" s="16">
+        <f>IFERROR(产品SKU!B8,"")</f>
+        <v/>
+      </c>
+      <c r="D80" s="16">
+        <f>IFERROR(产品SKU!D8,"")</f>
+        <v/>
+      </c>
+      <c r="E80" s="10">
+        <f>IFERROR(产品SKU!G8,0)</f>
+        <v/>
+      </c>
+      <c r="F80" s="10">
+        <f>IFERROR(过程品仓计算!E80/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G80" s="10">
+        <f>IFERROR(产品SKU!T8,0)</f>
+        <v/>
+      </c>
+      <c r="H80" s="10">
+        <f>IFERROR(过程品仓计算!F80*过程品仓计算!G80,0)</f>
+        <v/>
+      </c>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K80" s="10">
+        <f>IFERROR(IF(过程品仓计算!I80="",0,过程品仓计算!I80)*IF(过程品仓计算!J80="",0,过程品仓计算!J80),0)</f>
+        <v/>
+      </c>
+      <c r="L80" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H80,过程品仓计算!K80),0)</f>
+        <v/>
+      </c>
+      <c r="M80" s="9" t="n"/>
+      <c r="N80" s="9" t="n"/>
+      <c r="O80" s="9" t="n"/>
+      <c r="P80" s="10">
+        <f>IFERROR(过程品仓计算!L80+IF(过程品仓计算!M80="",0,过程品仓计算!M80)+IF(过程品仓计算!N80="",0,过程品仓计算!N80)+IF(过程品仓计算!O80="",0,过程品仓计算!O80),0)</f>
+        <v/>
+      </c>
+      <c r="Q80" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P80/MAX(产品SKU!M8,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="20" customHeight="1">
+      <c r="A81" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C81" s="16">
+        <f>IFERROR(产品SKU!B9,"")</f>
+        <v/>
+      </c>
+      <c r="D81" s="16">
+        <f>IFERROR(产品SKU!D9,"")</f>
+        <v/>
+      </c>
+      <c r="E81" s="10">
+        <f>IFERROR(产品SKU!G9,0)</f>
+        <v/>
+      </c>
+      <c r="F81" s="10">
+        <f>IFERROR(过程品仓计算!E81/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G81" s="10">
+        <f>IFERROR(产品SKU!T9,0)</f>
+        <v/>
+      </c>
+      <c r="H81" s="10">
+        <f>IFERROR(过程品仓计算!F81*过程品仓计算!G81,0)</f>
+        <v/>
+      </c>
+      <c r="I81" s="9" t="n"/>
+      <c r="J81" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K81" s="10">
+        <f>IFERROR(IF(过程品仓计算!I81="",0,过程品仓计算!I81)*IF(过程品仓计算!J81="",0,过程品仓计算!J81),0)</f>
+        <v/>
+      </c>
+      <c r="L81" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H81,过程品仓计算!K81),0)</f>
+        <v/>
+      </c>
+      <c r="M81" s="9" t="n"/>
+      <c r="N81" s="9" t="n"/>
+      <c r="O81" s="9" t="n"/>
+      <c r="P81" s="10">
+        <f>IFERROR(过程品仓计算!L81+IF(过程品仓计算!M81="",0,过程品仓计算!M81)+IF(过程品仓计算!N81="",0,过程品仓计算!N81)+IF(过程品仓计算!O81="",0,过程品仓计算!O81),0)</f>
+        <v/>
+      </c>
+      <c r="Q81" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P81/MAX(产品SKU!M9,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="20" customHeight="1">
+      <c r="A82" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C82" s="16">
+        <f>IFERROR(产品SKU!B10,"")</f>
+        <v/>
+      </c>
+      <c r="D82" s="16">
+        <f>IFERROR(产品SKU!D10,"")</f>
+        <v/>
+      </c>
+      <c r="E82" s="10">
+        <f>IFERROR(产品SKU!G10,0)</f>
+        <v/>
+      </c>
+      <c r="F82" s="10">
+        <f>IFERROR(过程品仓计算!E82/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G82" s="10">
+        <f>IFERROR(产品SKU!T10,0)</f>
+        <v/>
+      </c>
+      <c r="H82" s="10">
+        <f>IFERROR(过程品仓计算!F82*过程品仓计算!G82,0)</f>
+        <v/>
+      </c>
+      <c r="I82" s="9" t="n"/>
+      <c r="J82" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K82" s="10">
+        <f>IFERROR(IF(过程品仓计算!I82="",0,过程品仓计算!I82)*IF(过程品仓计算!J82="",0,过程品仓计算!J82),0)</f>
+        <v/>
+      </c>
+      <c r="L82" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H82,过程品仓计算!K82),0)</f>
+        <v/>
+      </c>
+      <c r="M82" s="9" t="n"/>
+      <c r="N82" s="9" t="n"/>
+      <c r="O82" s="9" t="n"/>
+      <c r="P82" s="10">
+        <f>IFERROR(过程品仓计算!L82+IF(过程品仓计算!M82="",0,过程品仓计算!M82)+IF(过程品仓计算!N82="",0,过程品仓计算!N82)+IF(过程品仓计算!O82="",0,过程品仓计算!O82),0)</f>
+        <v/>
+      </c>
+      <c r="Q82" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P82/MAX(产品SKU!M10,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C83" s="16">
+        <f>IFERROR(产品SKU!B11,"")</f>
+        <v/>
+      </c>
+      <c r="D83" s="16">
+        <f>IFERROR(产品SKU!D11,"")</f>
+        <v/>
+      </c>
+      <c r="E83" s="10">
+        <f>IFERROR(产品SKU!G11,0)</f>
+        <v/>
+      </c>
+      <c r="F83" s="10">
+        <f>IFERROR(过程品仓计算!E83/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G83" s="10">
+        <f>IFERROR(产品SKU!T11,0)</f>
+        <v/>
+      </c>
+      <c r="H83" s="10">
+        <f>IFERROR(过程品仓计算!F83*过程品仓计算!G83,0)</f>
+        <v/>
+      </c>
+      <c r="I83" s="9" t="n"/>
+      <c r="J83" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K83" s="10">
+        <f>IFERROR(IF(过程品仓计算!I83="",0,过程品仓计算!I83)*IF(过程品仓计算!J83="",0,过程品仓计算!J83),0)</f>
+        <v/>
+      </c>
+      <c r="L83" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H83,过程品仓计算!K83),0)</f>
+        <v/>
+      </c>
+      <c r="M83" s="9" t="n"/>
+      <c r="N83" s="9" t="n"/>
+      <c r="O83" s="9" t="n"/>
+      <c r="P83" s="10">
+        <f>IFERROR(过程品仓计算!L83+IF(过程品仓计算!M83="",0,过程品仓计算!M83)+IF(过程品仓计算!N83="",0,过程品仓计算!N83)+IF(过程品仓计算!O83="",0,过程品仓计算!O83),0)</f>
+        <v/>
+      </c>
+      <c r="Q83" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P83/MAX(产品SKU!M11,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" ht="20" customHeight="1">
+      <c r="A84" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C84" s="16">
+        <f>IFERROR(产品SKU!B12,"")</f>
+        <v/>
+      </c>
+      <c r="D84" s="16">
+        <f>IFERROR(产品SKU!D12,"")</f>
+        <v/>
+      </c>
+      <c r="E84" s="10">
+        <f>IFERROR(产品SKU!G12,0)</f>
+        <v/>
+      </c>
+      <c r="F84" s="10">
+        <f>IFERROR(过程品仓计算!E84/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G84" s="10">
+        <f>IFERROR(产品SKU!T12,0)</f>
+        <v/>
+      </c>
+      <c r="H84" s="10">
+        <f>IFERROR(过程品仓计算!F84*过程品仓计算!G84,0)</f>
+        <v/>
+      </c>
+      <c r="I84" s="9" t="n"/>
+      <c r="J84" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K84" s="10">
+        <f>IFERROR(IF(过程品仓计算!I84="",0,过程品仓计算!I84)*IF(过程品仓计算!J84="",0,过程品仓计算!J84),0)</f>
+        <v/>
+      </c>
+      <c r="L84" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H84,过程品仓计算!K84),0)</f>
+        <v/>
+      </c>
+      <c r="M84" s="9" t="n"/>
+      <c r="N84" s="9" t="n"/>
+      <c r="O84" s="9" t="n"/>
+      <c r="P84" s="10">
+        <f>IFERROR(过程品仓计算!L84+IF(过程品仓计算!M84="",0,过程品仓计算!M84)+IF(过程品仓计算!N84="",0,过程品仓计算!N84)+IF(过程品仓计算!O84="",0,过程品仓计算!O84),0)</f>
+        <v/>
+      </c>
+      <c r="Q84" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P84/MAX(产品SKU!M12,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="20" customHeight="1">
+      <c r="A85" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C85" s="16">
+        <f>IFERROR(产品SKU!B13,"")</f>
+        <v/>
+      </c>
+      <c r="D85" s="16">
+        <f>IFERROR(产品SKU!D13,"")</f>
+        <v/>
+      </c>
+      <c r="E85" s="10">
+        <f>IFERROR(产品SKU!G13,0)</f>
+        <v/>
+      </c>
+      <c r="F85" s="10">
+        <f>IFERROR(过程品仓计算!E85/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G85" s="10">
+        <f>IFERROR(产品SKU!T13,0)</f>
+        <v/>
+      </c>
+      <c r="H85" s="10">
+        <f>IFERROR(过程品仓计算!F85*过程品仓计算!G85,0)</f>
+        <v/>
+      </c>
+      <c r="I85" s="9" t="n"/>
+      <c r="J85" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K85" s="10">
+        <f>IFERROR(IF(过程品仓计算!I85="",0,过程品仓计算!I85)*IF(过程品仓计算!J85="",0,过程品仓计算!J85),0)</f>
+        <v/>
+      </c>
+      <c r="L85" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H85,过程品仓计算!K85),0)</f>
+        <v/>
+      </c>
+      <c r="M85" s="9" t="n"/>
+      <c r="N85" s="9" t="n"/>
+      <c r="O85" s="9" t="n"/>
+      <c r="P85" s="10">
+        <f>IFERROR(过程品仓计算!L85+IF(过程品仓计算!M85="",0,过程品仓计算!M85)+IF(过程品仓计算!N85="",0,过程品仓计算!N85)+IF(过程品仓计算!O85="",0,过程品仓计算!O85),0)</f>
+        <v/>
+      </c>
+      <c r="Q85" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P85/MAX(产品SKU!M13,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="A86" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存</t>
+        </is>
+      </c>
+      <c r="C86" s="16">
+        <f>IFERROR(产品SKU!B14,"")</f>
+        <v/>
+      </c>
+      <c r="D86" s="16">
+        <f>IFERROR(产品SKU!D14,"")</f>
+        <v/>
+      </c>
+      <c r="E86" s="10">
+        <f>IFERROR(产品SKU!G14,0)</f>
+        <v/>
+      </c>
+      <c r="F86" s="10">
+        <f>IFERROR(过程品仓计算!E86/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G86" s="10">
+        <f>IFERROR(产品SKU!T14,0)</f>
+        <v/>
+      </c>
+      <c r="H86" s="10">
+        <f>IFERROR(过程品仓计算!F86*过程品仓计算!G86,0)</f>
+        <v/>
+      </c>
+      <c r="I86" s="9" t="n"/>
+      <c r="J86" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K86" s="10">
+        <f>IFERROR(IF(过程品仓计算!I86="",0,过程品仓计算!I86)*IF(过程品仓计算!J86="",0,过程品仓计算!J86),0)</f>
+        <v/>
+      </c>
+      <c r="L86" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H86,过程品仓计算!K86),0)</f>
+        <v/>
+      </c>
+      <c r="M86" s="9" t="n"/>
+      <c r="N86" s="9" t="n"/>
+      <c r="O86" s="9" t="n"/>
+      <c r="P86" s="10">
+        <f>IFERROR(过程品仓计算!L86+IF(过程品仓计算!M86="",0,过程品仓计算!M86)+IF(过程品仓计算!N86="",0,过程品仓计算!N86)+IF(过程品仓计算!O86="",0,过程品仓计算!O86),0)</f>
+        <v/>
+      </c>
+      <c r="Q86" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P86/MAX(产品SKU!M14,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" ht="20" customHeight="1">
+      <c r="A87" s="19" t="inlineStr">
+        <is>
+          <t>高温碳化后暂存 小计</t>
+        </is>
+      </c>
+      <c r="P87" s="10">
+        <f>SUM(P75:P86)</f>
+        <v/>
+      </c>
+      <c r="Q87" s="10">
+        <f>SUM(Q75:Q86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>【成品筛分后暂存（成品前）】</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="20" customHeight="1">
+      <c r="A89" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C89" s="16">
+        <f>IFERROR(产品SKU!B3,"")</f>
+        <v/>
+      </c>
+      <c r="D89" s="16">
+        <f>IFERROR(产品SKU!D3,"")</f>
+        <v/>
+      </c>
+      <c r="E89" s="10">
+        <f>IFERROR(产品SKU!G3,0)</f>
+        <v/>
+      </c>
+      <c r="F89" s="10">
+        <f>IFERROR(过程品仓计算!E89/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G89" s="10">
+        <f>IFERROR(产品SKU!U3,0)</f>
+        <v/>
+      </c>
+      <c r="H89" s="10">
+        <f>IFERROR(过程品仓计算!F89*过程品仓计算!G89,0)</f>
+        <v/>
+      </c>
+      <c r="I89" s="9" t="n"/>
+      <c r="J89" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K89" s="10">
+        <f>IFERROR(IF(过程品仓计算!I89="",0,过程品仓计算!I89)*IF(过程品仓计算!J89="",0,过程品仓计算!J89),0)</f>
+        <v/>
+      </c>
+      <c r="L89" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H89,过程品仓计算!K89),0)</f>
+        <v/>
+      </c>
+      <c r="M89" s="9" t="n"/>
+      <c r="N89" s="9" t="n"/>
+      <c r="O89" s="9" t="n"/>
+      <c r="P89" s="10">
+        <f>IFERROR(过程品仓计算!L89+IF(过程品仓计算!M89="",0,过程品仓计算!M89)+IF(过程品仓计算!N89="",0,过程品仓计算!N89)+IF(过程品仓计算!O89="",0,过程品仓计算!O89),0)</f>
+        <v/>
+      </c>
+      <c r="Q89" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P89/MAX(产品SKU!M3,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="A90" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C90" s="16">
+        <f>IFERROR(产品SKU!B4,"")</f>
+        <v/>
+      </c>
+      <c r="D90" s="16">
+        <f>IFERROR(产品SKU!D4,"")</f>
+        <v/>
+      </c>
+      <c r="E90" s="10">
+        <f>IFERROR(产品SKU!G4,0)</f>
+        <v/>
+      </c>
+      <c r="F90" s="10">
+        <f>IFERROR(过程品仓计算!E90/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G90" s="10">
+        <f>IFERROR(产品SKU!U4,0)</f>
+        <v/>
+      </c>
+      <c r="H90" s="10">
+        <f>IFERROR(过程品仓计算!F90*过程品仓计算!G90,0)</f>
+        <v/>
+      </c>
+      <c r="I90" s="9" t="n"/>
+      <c r="J90" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K90" s="10">
+        <f>IFERROR(IF(过程品仓计算!I90="",0,过程品仓计算!I90)*IF(过程品仓计算!J90="",0,过程品仓计算!J90),0)</f>
+        <v/>
+      </c>
+      <c r="L90" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H90,过程品仓计算!K90),0)</f>
+        <v/>
+      </c>
+      <c r="M90" s="9" t="n"/>
+      <c r="N90" s="9" t="n"/>
+      <c r="O90" s="9" t="n"/>
+      <c r="P90" s="10">
+        <f>IFERROR(过程品仓计算!L90+IF(过程品仓计算!M90="",0,过程品仓计算!M90)+IF(过程品仓计算!N90="",0,过程品仓计算!N90)+IF(过程品仓计算!O90="",0,过程品仓计算!O90),0)</f>
+        <v/>
+      </c>
+      <c r="Q90" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P90/MAX(产品SKU!M4,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" ht="20" customHeight="1">
+      <c r="A91" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C91" s="16">
+        <f>IFERROR(产品SKU!B5,"")</f>
+        <v/>
+      </c>
+      <c r="D91" s="16">
+        <f>IFERROR(产品SKU!D5,"")</f>
+        <v/>
+      </c>
+      <c r="E91" s="10">
+        <f>IFERROR(产品SKU!G5,0)</f>
+        <v/>
+      </c>
+      <c r="F91" s="10">
+        <f>IFERROR(过程品仓计算!E91/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G91" s="10">
+        <f>IFERROR(产品SKU!U5,0)</f>
+        <v/>
+      </c>
+      <c r="H91" s="10">
+        <f>IFERROR(过程品仓计算!F91*过程品仓计算!G91,0)</f>
+        <v/>
+      </c>
+      <c r="I91" s="9" t="n"/>
+      <c r="J91" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K91" s="10">
+        <f>IFERROR(IF(过程品仓计算!I91="",0,过程品仓计算!I91)*IF(过程品仓计算!J91="",0,过程品仓计算!J91),0)</f>
+        <v/>
+      </c>
+      <c r="L91" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H91,过程品仓计算!K91),0)</f>
+        <v/>
+      </c>
+      <c r="M91" s="9" t="n"/>
+      <c r="N91" s="9" t="n"/>
+      <c r="O91" s="9" t="n"/>
+      <c r="P91" s="10">
+        <f>IFERROR(过程品仓计算!L91+IF(过程品仓计算!M91="",0,过程品仓计算!M91)+IF(过程品仓计算!N91="",0,过程品仓计算!N91)+IF(过程品仓计算!O91="",0,过程品仓计算!O91),0)</f>
+        <v/>
+      </c>
+      <c r="Q91" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P91/MAX(产品SKU!M5,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" ht="20" customHeight="1">
+      <c r="A92" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C92" s="16">
+        <f>IFERROR(产品SKU!B6,"")</f>
+        <v/>
+      </c>
+      <c r="D92" s="16">
+        <f>IFERROR(产品SKU!D6,"")</f>
+        <v/>
+      </c>
+      <c r="E92" s="10">
+        <f>IFERROR(产品SKU!G6,0)</f>
+        <v/>
+      </c>
+      <c r="F92" s="10">
+        <f>IFERROR(过程品仓计算!E92/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G92" s="10">
+        <f>IFERROR(产品SKU!U6,0)</f>
+        <v/>
+      </c>
+      <c r="H92" s="10">
+        <f>IFERROR(过程品仓计算!F92*过程品仓计算!G92,0)</f>
+        <v/>
+      </c>
+      <c r="I92" s="9" t="n"/>
+      <c r="J92" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K92" s="10">
+        <f>IFERROR(IF(过程品仓计算!I92="",0,过程品仓计算!I92)*IF(过程品仓计算!J92="",0,过程品仓计算!J92),0)</f>
+        <v/>
+      </c>
+      <c r="L92" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H92,过程品仓计算!K92),0)</f>
+        <v/>
+      </c>
+      <c r="M92" s="9" t="n"/>
+      <c r="N92" s="9" t="n"/>
+      <c r="O92" s="9" t="n"/>
+      <c r="P92" s="10">
+        <f>IFERROR(过程品仓计算!L92+IF(过程品仓计算!M92="",0,过程品仓计算!M92)+IF(过程品仓计算!N92="",0,过程品仓计算!N92)+IF(过程品仓计算!O92="",0,过程品仓计算!O92),0)</f>
+        <v/>
+      </c>
+      <c r="Q92" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P92/MAX(产品SKU!M6,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="20" customHeight="1">
+      <c r="A93" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C93" s="16">
+        <f>IFERROR(产品SKU!B7,"")</f>
+        <v/>
+      </c>
+      <c r="D93" s="16">
+        <f>IFERROR(产品SKU!D7,"")</f>
+        <v/>
+      </c>
+      <c r="E93" s="10">
+        <f>IFERROR(产品SKU!G7,0)</f>
+        <v/>
+      </c>
+      <c r="F93" s="10">
+        <f>IFERROR(过程品仓计算!E93/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G93" s="10">
+        <f>IFERROR(产品SKU!U7,0)</f>
+        <v/>
+      </c>
+      <c r="H93" s="10">
+        <f>IFERROR(过程品仓计算!F93*过程品仓计算!G93,0)</f>
+        <v/>
+      </c>
+      <c r="I93" s="9" t="n"/>
+      <c r="J93" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K93" s="10">
+        <f>IFERROR(IF(过程品仓计算!I93="",0,过程品仓计算!I93)*IF(过程品仓计算!J93="",0,过程品仓计算!J93),0)</f>
+        <v/>
+      </c>
+      <c r="L93" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H93,过程品仓计算!K93),0)</f>
+        <v/>
+      </c>
+      <c r="M93" s="9" t="n"/>
+      <c r="N93" s="9" t="n"/>
+      <c r="O93" s="9" t="n"/>
+      <c r="P93" s="10">
+        <f>IFERROR(过程品仓计算!L93+IF(过程品仓计算!M93="",0,过程品仓计算!M93)+IF(过程品仓计算!N93="",0,过程品仓计算!N93)+IF(过程品仓计算!O93="",0,过程品仓计算!O93),0)</f>
+        <v/>
+      </c>
+      <c r="Q93" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P93/MAX(产品SKU!M7,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" ht="20" customHeight="1">
+      <c r="A94" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C94" s="16">
+        <f>IFERROR(产品SKU!B8,"")</f>
+        <v/>
+      </c>
+      <c r="D94" s="16">
+        <f>IFERROR(产品SKU!D8,"")</f>
+        <v/>
+      </c>
+      <c r="E94" s="10">
+        <f>IFERROR(产品SKU!G8,0)</f>
+        <v/>
+      </c>
+      <c r="F94" s="10">
+        <f>IFERROR(过程品仓计算!E94/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G94" s="10">
+        <f>IFERROR(产品SKU!U8,0)</f>
+        <v/>
+      </c>
+      <c r="H94" s="10">
+        <f>IFERROR(过程品仓计算!F94*过程品仓计算!G94,0)</f>
+        <v/>
+      </c>
+      <c r="I94" s="9" t="n"/>
+      <c r="J94" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K94" s="10">
+        <f>IFERROR(IF(过程品仓计算!I94="",0,过程品仓计算!I94)*IF(过程品仓计算!J94="",0,过程品仓计算!J94),0)</f>
+        <v/>
+      </c>
+      <c r="L94" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H94,过程品仓计算!K94),0)</f>
+        <v/>
+      </c>
+      <c r="M94" s="9" t="n"/>
+      <c r="N94" s="9" t="n"/>
+      <c r="O94" s="9" t="n"/>
+      <c r="P94" s="10">
+        <f>IFERROR(过程品仓计算!L94+IF(过程品仓计算!M94="",0,过程品仓计算!M94)+IF(过程品仓计算!N94="",0,过程品仓计算!N94)+IF(过程品仓计算!O94="",0,过程品仓计算!O94),0)</f>
+        <v/>
+      </c>
+      <c r="Q94" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P94/MAX(产品SKU!M8,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="20" customHeight="1">
+      <c r="A95" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C95" s="16">
+        <f>IFERROR(产品SKU!B9,"")</f>
+        <v/>
+      </c>
+      <c r="D95" s="16">
+        <f>IFERROR(产品SKU!D9,"")</f>
+        <v/>
+      </c>
+      <c r="E95" s="10">
+        <f>IFERROR(产品SKU!G9,0)</f>
+        <v/>
+      </c>
+      <c r="F95" s="10">
+        <f>IFERROR(过程品仓计算!E95/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G95" s="10">
+        <f>IFERROR(产品SKU!U9,0)</f>
+        <v/>
+      </c>
+      <c r="H95" s="10">
+        <f>IFERROR(过程品仓计算!F95*过程品仓计算!G95,0)</f>
+        <v/>
+      </c>
+      <c r="I95" s="9" t="n"/>
+      <c r="J95" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K95" s="10">
+        <f>IFERROR(IF(过程品仓计算!I95="",0,过程品仓计算!I95)*IF(过程品仓计算!J95="",0,过程品仓计算!J95),0)</f>
+        <v/>
+      </c>
+      <c r="L95" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H95,过程品仓计算!K95),0)</f>
+        <v/>
+      </c>
+      <c r="M95" s="9" t="n"/>
+      <c r="N95" s="9" t="n"/>
+      <c r="O95" s="9" t="n"/>
+      <c r="P95" s="10">
+        <f>IFERROR(过程品仓计算!L95+IF(过程品仓计算!M95="",0,过程品仓计算!M95)+IF(过程品仓计算!N95="",0,过程品仓计算!N95)+IF(过程品仓计算!O95="",0,过程品仓计算!O95),0)</f>
+        <v/>
+      </c>
+      <c r="Q95" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P95/MAX(产品SKU!M9,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" ht="20" customHeight="1">
+      <c r="A96" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C96" s="16">
+        <f>IFERROR(产品SKU!B10,"")</f>
+        <v/>
+      </c>
+      <c r="D96" s="16">
+        <f>IFERROR(产品SKU!D10,"")</f>
+        <v/>
+      </c>
+      <c r="E96" s="10">
+        <f>IFERROR(产品SKU!G10,0)</f>
+        <v/>
+      </c>
+      <c r="F96" s="10">
+        <f>IFERROR(过程品仓计算!E96/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G96" s="10">
+        <f>IFERROR(产品SKU!U10,0)</f>
+        <v/>
+      </c>
+      <c r="H96" s="10">
+        <f>IFERROR(过程品仓计算!F96*过程品仓计算!G96,0)</f>
+        <v/>
+      </c>
+      <c r="I96" s="9" t="n"/>
+      <c r="J96" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K96" s="10">
+        <f>IFERROR(IF(过程品仓计算!I96="",0,过程品仓计算!I96)*IF(过程品仓计算!J96="",0,过程品仓计算!J96),0)</f>
+        <v/>
+      </c>
+      <c r="L96" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H96,过程品仓计算!K96),0)</f>
+        <v/>
+      </c>
+      <c r="M96" s="9" t="n"/>
+      <c r="N96" s="9" t="n"/>
+      <c r="O96" s="9" t="n"/>
+      <c r="P96" s="10">
+        <f>IFERROR(过程品仓计算!L96+IF(过程品仓计算!M96="",0,过程品仓计算!M96)+IF(过程品仓计算!N96="",0,过程品仓计算!N96)+IF(过程品仓计算!O96="",0,过程品仓计算!O96),0)</f>
+        <v/>
+      </c>
+      <c r="Q96" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P96/MAX(产品SKU!M10,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="20" customHeight="1">
+      <c r="A97" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B97" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C97" s="16">
+        <f>IFERROR(产品SKU!B11,"")</f>
+        <v/>
+      </c>
+      <c r="D97" s="16">
+        <f>IFERROR(产品SKU!D11,"")</f>
+        <v/>
+      </c>
+      <c r="E97" s="10">
+        <f>IFERROR(产品SKU!G11,0)</f>
+        <v/>
+      </c>
+      <c r="F97" s="10">
+        <f>IFERROR(过程品仓计算!E97/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G97" s="10">
+        <f>IFERROR(产品SKU!U11,0)</f>
+        <v/>
+      </c>
+      <c r="H97" s="10">
+        <f>IFERROR(过程品仓计算!F97*过程品仓计算!G97,0)</f>
+        <v/>
+      </c>
+      <c r="I97" s="9" t="n"/>
+      <c r="J97" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K97" s="10">
+        <f>IFERROR(IF(过程品仓计算!I97="",0,过程品仓计算!I97)*IF(过程品仓计算!J97="",0,过程品仓计算!J97),0)</f>
+        <v/>
+      </c>
+      <c r="L97" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H97,过程品仓计算!K97),0)</f>
+        <v/>
+      </c>
+      <c r="M97" s="9" t="n"/>
+      <c r="N97" s="9" t="n"/>
+      <c r="O97" s="9" t="n"/>
+      <c r="P97" s="10">
+        <f>IFERROR(过程品仓计算!L97+IF(过程品仓计算!M97="",0,过程品仓计算!M97)+IF(过程品仓计算!N97="",0,过程品仓计算!N97)+IF(过程品仓计算!O97="",0,过程品仓计算!O97),0)</f>
+        <v/>
+      </c>
+      <c r="Q97" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P97/MAX(产品SKU!M11,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" ht="20" customHeight="1">
+      <c r="A98" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="B98" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C98" s="16">
+        <f>IFERROR(产品SKU!B12,"")</f>
+        <v/>
+      </c>
+      <c r="D98" s="16">
+        <f>IFERROR(产品SKU!D12,"")</f>
+        <v/>
+      </c>
+      <c r="E98" s="10">
+        <f>IFERROR(产品SKU!G12,0)</f>
+        <v/>
+      </c>
+      <c r="F98" s="10">
+        <f>IFERROR(过程品仓计算!E98/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G98" s="10">
+        <f>IFERROR(产品SKU!U12,0)</f>
+        <v/>
+      </c>
+      <c r="H98" s="10">
+        <f>IFERROR(过程品仓计算!F98*过程品仓计算!G98,0)</f>
+        <v/>
+      </c>
+      <c r="I98" s="9" t="n"/>
+      <c r="J98" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K98" s="10">
+        <f>IFERROR(IF(过程品仓计算!I98="",0,过程品仓计算!I98)*IF(过程品仓计算!J98="",0,过程品仓计算!J98),0)</f>
+        <v/>
+      </c>
+      <c r="L98" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H98,过程品仓计算!K98),0)</f>
+        <v/>
+      </c>
+      <c r="M98" s="9" t="n"/>
+      <c r="N98" s="9" t="n"/>
+      <c r="O98" s="9" t="n"/>
+      <c r="P98" s="10">
+        <f>IFERROR(过程品仓计算!L98+IF(过程品仓计算!M98="",0,过程品仓计算!M98)+IF(过程品仓计算!N98="",0,过程品仓计算!N98)+IF(过程品仓计算!O98="",0,过程品仓计算!O98),0)</f>
+        <v/>
+      </c>
+      <c r="Q98" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P98/MAX(产品SKU!M12,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" ht="20" customHeight="1">
+      <c r="A99" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B99" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C99" s="16">
+        <f>IFERROR(产品SKU!B13,"")</f>
+        <v/>
+      </c>
+      <c r="D99" s="16">
+        <f>IFERROR(产品SKU!D13,"")</f>
+        <v/>
+      </c>
+      <c r="E99" s="10">
+        <f>IFERROR(产品SKU!G13,0)</f>
+        <v/>
+      </c>
+      <c r="F99" s="10">
+        <f>IFERROR(过程品仓计算!E99/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G99" s="10">
+        <f>IFERROR(产品SKU!U13,0)</f>
+        <v/>
+      </c>
+      <c r="H99" s="10">
+        <f>IFERROR(过程品仓计算!F99*过程品仓计算!G99,0)</f>
+        <v/>
+      </c>
+      <c r="I99" s="9" t="n"/>
+      <c r="J99" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K99" s="10">
+        <f>IFERROR(IF(过程品仓计算!I99="",0,过程品仓计算!I99)*IF(过程品仓计算!J99="",0,过程品仓计算!J99),0)</f>
+        <v/>
+      </c>
+      <c r="L99" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H99,过程品仓计算!K99),0)</f>
+        <v/>
+      </c>
+      <c r="M99" s="9" t="n"/>
+      <c r="N99" s="9" t="n"/>
+      <c r="O99" s="9" t="n"/>
+      <c r="P99" s="10">
+        <f>IFERROR(过程品仓计算!L99+IF(过程品仓计算!M99="",0,过程品仓计算!M99)+IF(过程品仓计算!N99="",0,过程品仓计算!N99)+IF(过程品仓计算!O99="",0,过程品仓计算!O99),0)</f>
+        <v/>
+      </c>
+      <c r="Q99" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P99/MAX(产品SKU!M13,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" ht="20" customHeight="1">
+      <c r="A100" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B100" s="16" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前）</t>
+        </is>
+      </c>
+      <c r="C100" s="16">
+        <f>IFERROR(产品SKU!B14,"")</f>
+        <v/>
+      </c>
+      <c r="D100" s="16">
+        <f>IFERROR(产品SKU!D14,"")</f>
+        <v/>
+      </c>
+      <c r="E100" s="10">
+        <f>IFERROR(产品SKU!G14,0)</f>
+        <v/>
+      </c>
+      <c r="F100" s="10">
+        <f>IFERROR(过程品仓计算!E100/参数设置!$C$5,0)</f>
+        <v/>
+      </c>
+      <c r="G100" s="10">
+        <f>IFERROR(产品SKU!U14,0)</f>
+        <v/>
+      </c>
+      <c r="H100" s="10">
+        <f>IFERROR(过程品仓计算!F100*过程品仓计算!G100,0)</f>
+        <v/>
+      </c>
+      <c r="I100" s="9" t="n"/>
+      <c r="J100" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K100" s="10">
+        <f>IFERROR(IF(过程品仓计算!I100="",0,过程品仓计算!I100)*IF(过程品仓计算!J100="",0,过程品仓计算!J100),0)</f>
+        <v/>
+      </c>
+      <c r="L100" s="10">
+        <f>IFERROR(MAX(过程品仓计算!H100,过程品仓计算!K100),0)</f>
+        <v/>
+      </c>
+      <c r="M100" s="9" t="n"/>
+      <c r="N100" s="9" t="n"/>
+      <c r="O100" s="9" t="n"/>
+      <c r="P100" s="10">
+        <f>IFERROR(过程品仓计算!L100+IF(过程品仓计算!M100="",0,过程品仓计算!M100)+IF(过程品仓计算!N100="",0,过程品仓计算!N100)+IF(过程品仓计算!O100="",0,过程品仓计算!O100),0)</f>
+        <v/>
+      </c>
+      <c r="Q100" s="10">
+        <f>IFERROR(CEILING(过程品仓计算!P100/MAX(产品SKU!M14,1),1)*参数设置!$C$13/MAX(参数设置!$C$14,1)/参数设置!$C$18*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" ht="20" customHeight="1">
+      <c r="A101" s="19" t="inlineStr">
+        <is>
+          <t>成品筛分后暂存（成品前） 小计</t>
+        </is>
+      </c>
+      <c r="P101" s="10">
+        <f>SUM(P89:P100)</f>
+        <v/>
+      </c>
+      <c r="Q101" s="10">
+        <f>SUM(Q89:Q100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="18" t="inlineStr">
         <is>
           <t>过程品仓 合计</t>
         </is>
       </c>
-      <c r="P46" s="10">
-        <f>SUMPRODUCT((MOD(ROW(P4:P45)-4,14)=(13))*P4:P45)</f>
-        <v/>
-      </c>
-      <c r="Q46" s="10">
-        <f>SUMPRODUCT((MOD(ROW(Q4:Q45)-4,14)=(13))*Q4:Q45)</f>
+      <c r="P102" s="10">
+        <f>SUMPRODUCT((MOD(ROW(P4:P101)-4,14)=(13))*P4:P101)</f>
+        <v/>
+      </c>
+      <c r="Q102" s="10">
+        <f>SUMPRODUCT((MOD(ROW(Q4:Q101)-4,14)=(13))*Q4:Q101)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="17">
+    <mergeCell ref="A87:O87"/>
+    <mergeCell ref="A59:O59"/>
+    <mergeCell ref="A74:Q74"/>
+    <mergeCell ref="A88:Q88"/>
     <mergeCell ref="A18:Q18"/>
+    <mergeCell ref="A73:O73"/>
+    <mergeCell ref="A101:O101"/>
     <mergeCell ref="A4:Q4"/>
+    <mergeCell ref="A102:O102"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="A45:O45"/>
-    <mergeCell ref="A46:O46"/>
     <mergeCell ref="A31:O31"/>
+    <mergeCell ref="A60:Q60"/>
     <mergeCell ref="A17:O17"/>
     <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A46:Q46"/>
     <mergeCell ref="A32:Q32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6656,7 +9632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -6761,7 +9737,7 @@
       <c r="A4" s="21" t="inlineStr">
         <is>
           <t>过程品仓
-（工序1后）</t>
+（粗破后）</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -6793,7 +9769,7 @@
       <c r="A5" s="20" t="inlineStr">
         <is>
           <t>过程品仓
-（工序2后）</t>
+（烘干后）</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -6825,7 +9801,7 @@
       <c r="A6" s="21" t="inlineStr">
         <is>
           <t>过程品仓
-（工序3后）</t>
+（磨粉后）</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -6854,18 +9830,19 @@
       <c r="H6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="22" t="inlineStr">
-        <is>
-          <t>过程品仓 合计</t>
+      <c r="A7" s="20" t="inlineStr">
+        <is>
+          <t>过程品仓
+（低温碳化后）</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>见过程品仓计算!P46</t>
+          <t>MAX(下游小时消耗×缓冲小时数, 批量×等待批次) + 待检 + 尾批 + 不良品</t>
         </is>
       </c>
       <c r="C7" s="10">
-        <f>过程品仓计算!P46</f>
+        <f>过程品仓计算!P59</f>
         <v/>
       </c>
       <c r="D7" s="8" t="inlineStr">
@@ -6875,7 +9852,7 @@
       </c>
       <c r="E7" s="9" t="n"/>
       <c r="F7" s="10">
-        <f>过程品仓计算!Q46</f>
+        <f>过程品仓计算!Q59</f>
         <v/>
       </c>
       <c r="G7" s="10">
@@ -6887,16 +9864,17 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>成品仓</t>
+          <t>过程品仓
+（石墨化后）</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>MAX(日需求×生产间隔, 日需求×目标天数, 最小批量) + 安全库存 + 待检放行</t>
+          <t>MAX(下游小时消耗×缓冲小时数, 批量×等待批次) + 待检 + 尾批 + 不良品</t>
         </is>
       </c>
       <c r="C8" s="10">
-        <f>成品仓计算!N16</f>
+        <f>过程品仓计算!P73</f>
         <v/>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -6906,7 +9884,7 @@
       </c>
       <c r="E8" s="9" t="n"/>
       <c r="F8" s="10">
-        <f>成品仓计算!O16</f>
+        <f>过程品仓计算!Q73</f>
         <v/>
       </c>
       <c r="G8" s="10">
@@ -6915,102 +9893,228 @@
       </c>
       <c r="H8" s="8" t="inlineStr"/>
     </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>过程品仓
+（高温碳化后）</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>MAX(下游小时消耗×缓冲小时数, 批量×等待批次) + 待检 + 尾批 + 不良品</t>
+        </is>
+      </c>
+      <c r="C9" s="10">
+        <f>过程品仓计算!P87</f>
+        <v/>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n"/>
+      <c r="F9" s="10">
+        <f>过程品仓计算!Q87</f>
+        <v/>
+      </c>
+      <c r="G9" s="10">
+        <f>IFERROR(汇总!F9*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>过程品仓
+（成品筛分后）</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>MAX(下游小时消耗×缓冲小时数, 批量×等待批次) + 待检 + 尾批 + 不良品</t>
+        </is>
+      </c>
+      <c r="C10" s="10">
+        <f>过程品仓计算!P101</f>
+        <v/>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="n"/>
+      <c r="F10" s="10">
+        <f>过程品仓计算!Q101</f>
+        <v/>
+      </c>
+      <c r="G10" s="10">
+        <f>IFERROR(汇总!F10*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="8" t="inlineStr"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>过程品仓 合计</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>见过程品仓计算!P102</t>
+        </is>
+      </c>
+      <c r="C11" s="10">
+        <f>过程品仓计算!P102</f>
+        <v/>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="n"/>
+      <c r="F11" s="10">
+        <f>过程品仓计算!Q102</f>
+        <v/>
+      </c>
+      <c r="G11" s="10">
+        <f>IFERROR(汇总!F11*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>成品仓</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>MAX(日需求×生产间隔, 日需求×目标天数, 最小批量) + 安全库存 + 待检放行</t>
+        </is>
+      </c>
+      <c r="C12" s="10">
+        <f>成品仓计算!N16</f>
+        <v/>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>件</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="10">
+        <f>成品仓计算!O16</f>
+        <v/>
+      </c>
+      <c r="G12" s="10">
+        <f>IFERROR(汇总!F12*参数设置!$C$21,0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>三类仓库合计（不含辅助区域）</t>
         </is>
       </c>
-      <c r="G9" s="10">
-        <f>IFERROR(汇总!G3+汇总!G7+汇总!G8,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="G13" s="10">
+        <f>IFERROR(汇总!G3+汇总!G11+汇总!G12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>⚠ 上述面积为存储区估算，实际仓库还需加上：收发货区、质检区、不良品隔离区、退换货区、包装区、通道等辅助区域，通常再增加30%~50%的辅助面积。</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="25" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
         <is>
           <t>★ 面积估算关键参数(可在[参数设置]工作表中修改)：</t>
         </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>单托盘占地面积</t>
-        </is>
-      </c>
-      <c r="B14" s="16">
-        <f>参数设置!C13&amp;" m²"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>地堆层数</t>
-        </is>
-      </c>
-      <c r="B15" s="16">
-        <f>参数设置!C14&amp;" 层"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>原料仓面积利用率</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>TEXT(参数设置!C17,"0.0%")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>过程品仓面积利用率</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>TEXT(参数设置!C18,"0.0%")</f>
-        <v/>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>成品仓面积利用率</t>
+          <t>单托盘占地面积</t>
         </is>
       </c>
       <c r="B18" s="16">
-        <f>TEXT(参数设置!C19,"0.0%")</f>
+        <f>参数设置!C13&amp;" m²"</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
+          <t>地堆层数</t>
+        </is>
+      </c>
+      <c r="B19" s="16">
+        <f>参数设置!C14&amp;" 层"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>原料仓面积利用率</t>
+        </is>
+      </c>
+      <c r="B20" s="16">
+        <f>TEXT(参数设置!C17,"0.0%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>过程品仓面积利用率</t>
+        </is>
+      </c>
+      <c r="B21" s="16">
+        <f>TEXT(参数设置!C18,"0.0%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>成品仓面积利用率</t>
+        </is>
+      </c>
+      <c r="B22" s="16">
+        <f>TEXT(参数设置!C19,"0.0%")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
           <t>扩展余量系数</t>
         </is>
       </c>
-      <c r="B19" s="16">
+      <c r="B23" s="16">
         <f>参数设置!C21</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A17:H17"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>